<commit_message>
Set up Full Docker
</commit_message>
<xml_diff>
--- a/src/test/resources/data/User_Data.xlsx
+++ b/src/test/resources/data/User_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Zalo\DATN\Automation_AFF\src\test\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22AA3D40-708D-4630-A562-53999C7F585F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E8C2E35-2D28-45A3-A84F-E9289273895D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="330" yWindow="-120" windowWidth="28590" windowHeight="16440" tabRatio="920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="730">
   <si>
     <t>Cần để ý :</t>
   </si>
@@ -2253,6 +2253,42 @@
   </si>
   <si>
     <t>Khi code thêm 1 rồi xem có giảm về 0 được không</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4200</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4201</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4202</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4203</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4204</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4205</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4206</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4207</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4208</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4209</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4210</t>
+  </si>
+  <si>
+    <t>127.0.0.1/4211</t>
   </si>
 </sst>
 </file>
@@ -2310,13 +2346,6 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Times New Roman"/>
@@ -2393,6 +2422,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2421,7 +2456,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2523,89 +2558,86 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="16" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2617,17 +2649,17 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2970,25 +3002,25 @@
       </c>
     </row>
     <row r="2" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="40" t="s">
+      <c r="C2" s="39" t="s">
         <v>661</v>
       </c>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="38" t="s">
         <v>479</v>
       </c>
-      <c r="E2" s="41" t="s">
-        <v>557</v>
-      </c>
-      <c r="F2" s="39" t="s">
+      <c r="E2" s="40" t="s">
+        <v>718</v>
+      </c>
+      <c r="F2" s="38" t="s">
         <v>662</v>
       </c>
-      <c r="G2" s="39" t="s">
+      <c r="G2" s="38" t="s">
         <v>504</v>
       </c>
     </row>
@@ -3003,8 +3035,8 @@
       <c r="D3" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="E3" s="36" t="s">
-        <v>557</v>
+      <c r="E3" s="40" t="s">
+        <v>719</v>
       </c>
       <c r="F3" s="34" t="s">
         <v>481</v>
@@ -3026,8 +3058,8 @@
       <c r="D4" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="E4" s="36" t="s">
-        <v>557</v>
+      <c r="E4" s="40" t="s">
+        <v>720</v>
       </c>
       <c r="F4" s="34" t="s">
         <v>484</v>
@@ -3049,8 +3081,8 @@
       <c r="D5" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="E5" s="36" t="s">
-        <v>557</v>
+      <c r="E5" s="40" t="s">
+        <v>721</v>
       </c>
       <c r="F5" s="34" t="s">
         <v>485</v>
@@ -3072,8 +3104,8 @@
       <c r="D6" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="E6" s="36" t="s">
-        <v>557</v>
+      <c r="E6" s="40" t="s">
+        <v>722</v>
       </c>
       <c r="F6" s="34" t="s">
         <v>486</v>
@@ -3095,8 +3127,8 @@
       <c r="D7" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="E7" s="36" t="s">
-        <v>557</v>
+      <c r="E7" s="40" t="s">
+        <v>723</v>
       </c>
       <c r="F7" s="34" t="s">
         <v>487</v>
@@ -3118,8 +3150,8 @@
       <c r="D8" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="E8" s="36" t="s">
-        <v>557</v>
+      <c r="E8" s="40" t="s">
+        <v>724</v>
       </c>
       <c r="F8" s="34" t="s">
         <v>488</v>
@@ -3141,8 +3173,8 @@
       <c r="D9" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="E9" s="36" t="s">
-        <v>557</v>
+      <c r="E9" s="40" t="s">
+        <v>725</v>
       </c>
       <c r="F9" s="34" t="s">
         <v>489</v>
@@ -3164,8 +3196,8 @@
       <c r="D10" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="E10" s="36" t="s">
-        <v>557</v>
+      <c r="E10" s="40" t="s">
+        <v>726</v>
       </c>
       <c r="F10" s="34" t="s">
         <v>670</v>
@@ -3178,15 +3210,15 @@
       <c r="A11" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="37"/>
+      <c r="B11" s="36"/>
       <c r="C11" s="35" t="s">
         <v>631</v>
       </c>
       <c r="D11" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="E11" s="36" t="s">
-        <v>557</v>
+      <c r="E11" s="40" t="s">
+        <v>727</v>
       </c>
       <c r="F11" s="34" t="s">
         <v>632</v>
@@ -3208,8 +3240,8 @@
       <c r="D12" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="E12" s="36" t="s">
-        <v>557</v>
+      <c r="E12" s="40" t="s">
+        <v>728</v>
       </c>
       <c r="F12" s="34" t="s">
         <v>636</v>
@@ -3231,8 +3263,8 @@
       <c r="D13" s="34" t="s">
         <v>479</v>
       </c>
-      <c r="E13" s="36" t="s">
-        <v>557</v>
+      <c r="E13" s="40" t="s">
+        <v>729</v>
       </c>
       <c r="F13" s="34" t="s">
         <v>673</v>
@@ -3242,15 +3274,16 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="38"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="38"/>
-      <c r="G14" s="38"/>
+      <c r="A14" s="37"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="37"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3287,7 +3320,7 @@
       <c r="E1" s="20" t="s">
         <v>435</v>
       </c>
-      <c r="F1" s="64" t="s">
+      <c r="F1" s="63" t="s">
         <v>470</v>
       </c>
       <c r="G1" s="21" t="s">
@@ -3310,7 +3343,7 @@
       <c r="E2" s="20" t="s">
         <v>702</v>
       </c>
-      <c r="F2" s="64" t="s">
+      <c r="F2" s="63" t="s">
         <v>6</v>
       </c>
       <c r="G2" s="21" t="s">
@@ -3336,7 +3369,7 @@
       <c r="E3" s="20" t="s">
         <v>703</v>
       </c>
-      <c r="F3" s="64" t="s">
+      <c r="F3" s="63" t="s">
         <v>6</v>
       </c>
       <c r="G3" s="21" t="s">
@@ -3362,7 +3395,7 @@
       <c r="E4" s="20" t="s">
         <v>453</v>
       </c>
-      <c r="F4" s="64" t="s">
+      <c r="F4" s="63" t="s">
         <v>482</v>
       </c>
       <c r="G4" s="21" t="s">
@@ -3388,7 +3421,7 @@
     <col min="1" max="4" width="9.140625" style="21" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20" style="21" bestFit="1" customWidth="1"/>
     <col min="6" max="10" width="9.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="38" style="64" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="38" style="63" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="40.85546875" style="21" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="9.140625" style="21"/>
   </cols>
@@ -3409,20 +3442,20 @@
       <c r="E1" s="20" t="s">
         <v>435</v>
       </c>
-      <c r="F1" s="64" t="s">
+      <c r="F1" s="63" t="s">
         <v>470</v>
       </c>
       <c r="G1" s="21" t="s">
         <v>693</v>
       </c>
       <c r="K1" s="20"/>
-      <c r="L1" s="64"/>
+      <c r="L1" s="63"/>
     </row>
     <row r="2" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E2" s="20" t="s">
         <v>451</v>
       </c>
-      <c r="F2" s="64" t="s">
+      <c r="F2" s="63" t="s">
         <v>6</v>
       </c>
       <c r="G2" s="21" t="s">
@@ -3433,7 +3466,7 @@
       <c r="E3" s="20" t="s">
         <v>452</v>
       </c>
-      <c r="F3" s="64" t="s">
+      <c r="F3" s="63" t="s">
         <v>6</v>
       </c>
       <c r="G3" s="21" t="s">
@@ -3442,7 +3475,7 @@
     </row>
     <row r="4" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E4" s="20"/>
-      <c r="F4" s="64"/>
+      <c r="F4" s="63"/>
     </row>
     <row r="5" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3462,7 +3495,7 @@
     <row r="18" spans="11:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="11:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="11:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K20" s="65"/>
+      <c r="K20" s="64"/>
     </row>
     <row r="21" spans="11:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="22" spans="11:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3949,12 +3982,12 @@
         <v>8</v>
       </c>
       <c r="I15" s="6"/>
-      <c r="J15" s="70" t="s">
+      <c r="J15" s="68" t="s">
         <v>9</v>
       </c>
-      <c r="K15" s="70"/>
-      <c r="L15" s="70"/>
-      <c r="M15" s="70"/>
+      <c r="K15" s="68"/>
+      <c r="L15" s="68"/>
+      <c r="M15" s="68"/>
       <c r="N15" s="7"/>
       <c r="O15" s="8">
         <v>1</v>
@@ -3980,12 +4013,12 @@
         <v>14</v>
       </c>
       <c r="I16" s="6"/>
-      <c r="J16" s="70" t="s">
+      <c r="J16" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="K16" s="70"/>
-      <c r="L16" s="70"/>
-      <c r="M16" s="70"/>
+      <c r="K16" s="68"/>
+      <c r="L16" s="68"/>
+      <c r="M16" s="68"/>
       <c r="N16" s="7"/>
       <c r="O16" s="8">
         <v>50</v>
@@ -4006,12 +4039,12 @@
         <v>19</v>
       </c>
       <c r="I17" s="6"/>
-      <c r="J17" s="70" t="s">
+      <c r="J17" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="K17" s="70"/>
-      <c r="L17" s="70"/>
-      <c r="M17" s="70"/>
+      <c r="K17" s="68"/>
+      <c r="L17" s="68"/>
+      <c r="M17" s="68"/>
       <c r="N17" s="7"/>
       <c r="O17" s="8">
         <v>51</v>
@@ -4035,12 +4068,12 @@
         <v>25</v>
       </c>
       <c r="I18" s="6"/>
-      <c r="J18" s="70" t="s">
+      <c r="J18" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="K18" s="70"/>
-      <c r="L18" s="70"/>
-      <c r="M18" s="70"/>
+      <c r="K18" s="68"/>
+      <c r="L18" s="68"/>
+      <c r="M18" s="68"/>
       <c r="N18" s="7"/>
       <c r="O18" s="8">
         <v>52</v>
@@ -4058,12 +4091,12 @@
         <v>29</v>
       </c>
       <c r="I19" s="6"/>
-      <c r="J19" s="70" t="s">
+      <c r="J19" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="K19" s="70"/>
-      <c r="L19" s="70"/>
-      <c r="M19" s="70"/>
+      <c r="K19" s="68"/>
+      <c r="L19" s="68"/>
+      <c r="M19" s="68"/>
       <c r="N19" s="7"/>
       <c r="O19" s="8">
         <v>53</v>
@@ -4112,12 +4145,12 @@
       <c r="R21" s="6"/>
     </row>
     <row r="22" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="72" t="s">
+      <c r="B22" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="72"/>
-      <c r="D22" s="72"/>
-      <c r="E22" s="72"/>
+      <c r="C22" s="69"/>
+      <c r="D22" s="69"/>
+      <c r="E22" s="69"/>
       <c r="I22" s="6"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
@@ -4136,12 +4169,12 @@
       <c r="R22" s="6"/>
     </row>
     <row r="23" spans="2:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="72" t="s">
+      <c r="B23" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="72"/>
-      <c r="D23" s="72"/>
-      <c r="E23" s="72"/>
+      <c r="C23" s="69"/>
+      <c r="D23" s="69"/>
+      <c r="E23" s="69"/>
       <c r="F23" s="4" t="s">
         <v>42</v>
       </c>
@@ -4159,12 +4192,12 @@
       <c r="R23" s="6"/>
     </row>
     <row r="24" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="72" t="s">
+      <c r="B24" s="69" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="72"/>
-      <c r="D24" s="72"/>
-      <c r="E24" s="72"/>
+      <c r="C24" s="69"/>
+      <c r="D24" s="69"/>
+      <c r="E24" s="69"/>
       <c r="I24" s="6"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
@@ -4183,12 +4216,12 @@
       <c r="R24" s="6"/>
     </row>
     <row r="25" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="72" t="s">
+      <c r="B25" s="69" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="72"/>
-      <c r="D25" s="72"/>
-      <c r="E25" s="72"/>
+      <c r="C25" s="69"/>
+      <c r="D25" s="69"/>
+      <c r="E25" s="69"/>
       <c r="I25" s="6"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
@@ -4207,12 +4240,12 @@
       <c r="R25" s="6"/>
     </row>
     <row r="26" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="72" t="s">
+      <c r="B26" s="69" t="s">
         <v>51</v>
       </c>
-      <c r="C26" s="72"/>
-      <c r="D26" s="72"/>
-      <c r="E26" s="72"/>
+      <c r="C26" s="69"/>
+      <c r="D26" s="69"/>
+      <c r="E26" s="69"/>
       <c r="I26" s="6"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
@@ -4231,17 +4264,17 @@
       <c r="R26" s="6"/>
     </row>
     <row r="27" spans="2:18" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="72" t="s">
+      <c r="B27" s="69" t="s">
         <v>54</v>
       </c>
-      <c r="C27" s="72"/>
-      <c r="D27" s="72"/>
-      <c r="E27" s="72"/>
+      <c r="C27" s="69"/>
+      <c r="D27" s="69"/>
+      <c r="E27" s="69"/>
       <c r="I27" s="6"/>
-      <c r="J27" s="69"/>
-      <c r="K27" s="69"/>
-      <c r="L27" s="69"/>
-      <c r="M27" s="69"/>
+      <c r="J27" s="70"/>
+      <c r="K27" s="70"/>
+      <c r="L27" s="70"/>
+      <c r="M27" s="70"/>
       <c r="N27" s="7"/>
       <c r="O27" s="8">
         <v>61</v>
@@ -4255,17 +4288,17 @@
       <c r="R27" s="6"/>
     </row>
     <row r="28" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="72" t="s">
+      <c r="B28" s="69" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="72"/>
-      <c r="D28" s="72"/>
-      <c r="E28" s="72"/>
+      <c r="C28" s="69"/>
+      <c r="D28" s="69"/>
+      <c r="E28" s="69"/>
       <c r="I28" s="6"/>
-      <c r="J28" s="70"/>
-      <c r="K28" s="70"/>
-      <c r="L28" s="70"/>
-      <c r="M28" s="70"/>
+      <c r="J28" s="68"/>
+      <c r="K28" s="68"/>
+      <c r="L28" s="68"/>
+      <c r="M28" s="68"/>
       <c r="N28" s="9"/>
       <c r="O28" s="8">
         <v>62</v>
@@ -4280,10 +4313,10 @@
     </row>
     <row r="29" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I29" s="6"/>
-      <c r="J29" s="70"/>
-      <c r="K29" s="70"/>
-      <c r="L29" s="70"/>
-      <c r="M29" s="70"/>
+      <c r="J29" s="68"/>
+      <c r="K29" s="68"/>
+      <c r="L29" s="68"/>
+      <c r="M29" s="68"/>
       <c r="N29" s="9"/>
       <c r="O29" s="8">
         <v>63</v>
@@ -4298,10 +4331,10 @@
     </row>
     <row r="30" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I30" s="6"/>
-      <c r="J30" s="70"/>
-      <c r="K30" s="70"/>
-      <c r="L30" s="70"/>
-      <c r="M30" s="70"/>
+      <c r="J30" s="68"/>
+      <c r="K30" s="68"/>
+      <c r="L30" s="68"/>
+      <c r="M30" s="68"/>
       <c r="N30" s="9"/>
       <c r="O30" s="8">
         <v>64</v>
@@ -4316,10 +4349,10 @@
     </row>
     <row r="31" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I31" s="6"/>
-      <c r="J31" s="70"/>
-      <c r="K31" s="70"/>
-      <c r="L31" s="70"/>
-      <c r="M31" s="70"/>
+      <c r="J31" s="68"/>
+      <c r="K31" s="68"/>
+      <c r="L31" s="68"/>
+      <c r="M31" s="68"/>
       <c r="N31" s="9"/>
       <c r="O31" s="8">
         <v>65</v>
@@ -4334,10 +4367,10 @@
     </row>
     <row r="32" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I32" s="6"/>
-      <c r="J32" s="70"/>
-      <c r="K32" s="70"/>
-      <c r="L32" s="70"/>
-      <c r="M32" s="70"/>
+      <c r="J32" s="68"/>
+      <c r="K32" s="68"/>
+      <c r="L32" s="68"/>
+      <c r="M32" s="68"/>
       <c r="N32" s="9"/>
       <c r="O32" s="8">
         <v>66</v>
@@ -4352,10 +4385,10 @@
     </row>
     <row r="33" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I33" s="6"/>
-      <c r="J33" s="70"/>
-      <c r="K33" s="70"/>
-      <c r="L33" s="70"/>
-      <c r="M33" s="70"/>
+      <c r="J33" s="68"/>
+      <c r="K33" s="68"/>
+      <c r="L33" s="68"/>
+      <c r="M33" s="68"/>
       <c r="N33" s="9"/>
       <c r="O33" s="8">
         <v>67</v>
@@ -4370,10 +4403,10 @@
     </row>
     <row r="34" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I34" s="6"/>
-      <c r="J34" s="70"/>
-      <c r="K34" s="70"/>
-      <c r="L34" s="70"/>
-      <c r="M34" s="70"/>
+      <c r="J34" s="68"/>
+      <c r="K34" s="68"/>
+      <c r="L34" s="68"/>
+      <c r="M34" s="68"/>
       <c r="N34" s="9"/>
       <c r="O34" s="8">
         <v>68</v>
@@ -4388,10 +4421,10 @@
     </row>
     <row r="35" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I35" s="6"/>
-      <c r="J35" s="70"/>
-      <c r="K35" s="70"/>
-      <c r="L35" s="70"/>
-      <c r="M35" s="70"/>
+      <c r="J35" s="68"/>
+      <c r="K35" s="68"/>
+      <c r="L35" s="68"/>
+      <c r="M35" s="68"/>
       <c r="N35" s="9"/>
       <c r="O35" s="8">
         <v>69</v>
@@ -4406,10 +4439,10 @@
     </row>
     <row r="36" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I36" s="6"/>
-      <c r="J36" s="70"/>
-      <c r="K36" s="70"/>
-      <c r="L36" s="70"/>
-      <c r="M36" s="70"/>
+      <c r="J36" s="68"/>
+      <c r="K36" s="68"/>
+      <c r="L36" s="68"/>
+      <c r="M36" s="68"/>
       <c r="N36" s="9"/>
       <c r="O36" s="8">
         <v>70</v>
@@ -4427,10 +4460,10 @@
         <v>76</v>
       </c>
       <c r="I37" s="6"/>
-      <c r="J37" s="70"/>
-      <c r="K37" s="70"/>
-      <c r="L37" s="70"/>
-      <c r="M37" s="70"/>
+      <c r="J37" s="68"/>
+      <c r="K37" s="68"/>
+      <c r="L37" s="68"/>
+      <c r="M37" s="68"/>
       <c r="N37" s="9"/>
       <c r="O37" s="8">
         <v>71</v>
@@ -4445,10 +4478,10 @@
     </row>
     <row r="38" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I38" s="6"/>
-      <c r="J38" s="69"/>
-      <c r="K38" s="69"/>
-      <c r="L38" s="69"/>
-      <c r="M38" s="69"/>
+      <c r="J38" s="70"/>
+      <c r="K38" s="70"/>
+      <c r="L38" s="70"/>
+      <c r="M38" s="70"/>
       <c r="N38" s="9"/>
       <c r="O38" s="8">
         <v>72</v>
@@ -4463,10 +4496,10 @@
     </row>
     <row r="39" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I39" s="6"/>
-      <c r="J39" s="69"/>
-      <c r="K39" s="69"/>
-      <c r="L39" s="69"/>
-      <c r="M39" s="69"/>
+      <c r="J39" s="70"/>
+      <c r="K39" s="70"/>
+      <c r="L39" s="70"/>
+      <c r="M39" s="70"/>
       <c r="N39" s="9"/>
       <c r="O39" s="8">
         <v>73</v>
@@ -4481,10 +4514,10 @@
     </row>
     <row r="40" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I40" s="6"/>
-      <c r="J40" s="69"/>
-      <c r="K40" s="69"/>
-      <c r="L40" s="69"/>
-      <c r="M40" s="69"/>
+      <c r="J40" s="70"/>
+      <c r="K40" s="70"/>
+      <c r="L40" s="70"/>
+      <c r="M40" s="70"/>
       <c r="N40" s="7"/>
       <c r="O40" s="8">
         <v>74</v>
@@ -4499,10 +4532,10 @@
     </row>
     <row r="41" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I41" s="6"/>
-      <c r="J41" s="69"/>
-      <c r="K41" s="69"/>
-      <c r="L41" s="69"/>
-      <c r="M41" s="69"/>
+      <c r="J41" s="70"/>
+      <c r="K41" s="70"/>
+      <c r="L41" s="70"/>
+      <c r="M41" s="70"/>
       <c r="N41" s="7"/>
       <c r="O41" s="8">
         <v>75</v>
@@ -4517,12 +4550,12 @@
     </row>
     <row r="42" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I42" s="6"/>
-      <c r="J42" s="70" t="s">
+      <c r="J42" s="68" t="s">
         <v>86</v>
       </c>
-      <c r="K42" s="70"/>
-      <c r="L42" s="70"/>
-      <c r="M42" s="70"/>
+      <c r="K42" s="68"/>
+      <c r="L42" s="68"/>
+      <c r="M42" s="68"/>
       <c r="N42" s="9"/>
       <c r="O42" s="8">
         <v>76</v>
@@ -4537,12 +4570,12 @@
     </row>
     <row r="43" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I43" s="71"/>
-      <c r="J43" s="70" t="s">
+      <c r="J43" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="K43" s="70"/>
-      <c r="L43" s="70"/>
-      <c r="M43" s="70"/>
+      <c r="K43" s="68"/>
+      <c r="L43" s="68"/>
+      <c r="M43" s="68"/>
       <c r="N43" s="9"/>
       <c r="O43" s="8">
         <v>77</v>
@@ -4556,13 +4589,13 @@
       <c r="R43" s="6"/>
     </row>
     <row r="44" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I44" s="72"/>
-      <c r="J44" s="70" t="s">
+      <c r="I44" s="69"/>
+      <c r="J44" s="68" t="s">
         <v>92</v>
       </c>
-      <c r="K44" s="70"/>
-      <c r="L44" s="70"/>
-      <c r="M44" s="70"/>
+      <c r="K44" s="68"/>
+      <c r="L44" s="68"/>
+      <c r="M44" s="68"/>
       <c r="N44" s="9"/>
       <c r="O44" s="8">
         <v>78</v>
@@ -4576,13 +4609,13 @@
       <c r="R44" s="6"/>
     </row>
     <row r="45" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I45" s="72"/>
-      <c r="J45" s="70" t="s">
+      <c r="I45" s="69"/>
+      <c r="J45" s="68" t="s">
         <v>95</v>
       </c>
-      <c r="K45" s="70"/>
-      <c r="L45" s="70"/>
-      <c r="M45" s="70"/>
+      <c r="K45" s="68"/>
+      <c r="L45" s="68"/>
+      <c r="M45" s="68"/>
       <c r="N45" s="9"/>
       <c r="O45" s="8">
         <v>79</v>
@@ -4596,13 +4629,13 @@
       <c r="R45" s="6"/>
     </row>
     <row r="46" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I46" s="72"/>
-      <c r="J46" s="70" t="s">
+      <c r="I46" s="69"/>
+      <c r="J46" s="68" t="s">
         <v>98</v>
       </c>
-      <c r="K46" s="70"/>
-      <c r="L46" s="70"/>
-      <c r="M46" s="70"/>
+      <c r="K46" s="68"/>
+      <c r="L46" s="68"/>
+      <c r="M46" s="68"/>
       <c r="N46" s="9"/>
       <c r="O46" s="8">
         <v>80</v>
@@ -4616,13 +4649,13 @@
       <c r="R46" s="6"/>
     </row>
     <row r="47" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I47" s="72"/>
-      <c r="J47" s="70" t="s">
+      <c r="I47" s="69"/>
+      <c r="J47" s="68" t="s">
         <v>101</v>
       </c>
-      <c r="K47" s="70"/>
-      <c r="L47" s="70"/>
-      <c r="M47" s="70"/>
+      <c r="K47" s="68"/>
+      <c r="L47" s="68"/>
+      <c r="M47" s="68"/>
       <c r="N47" s="9"/>
       <c r="O47" s="8">
         <v>81</v>
@@ -4636,13 +4669,13 @@
       <c r="R47" s="6"/>
     </row>
     <row r="48" spans="2:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I48" s="72"/>
-      <c r="J48" s="70" t="s">
+      <c r="I48" s="69"/>
+      <c r="J48" s="68" t="s">
         <v>104</v>
       </c>
-      <c r="K48" s="70"/>
-      <c r="L48" s="70"/>
-      <c r="M48" s="70"/>
+      <c r="K48" s="68"/>
+      <c r="L48" s="68"/>
+      <c r="M48" s="68"/>
       <c r="N48" s="9"/>
       <c r="O48" s="8">
         <v>82</v>
@@ -4656,11 +4689,11 @@
       <c r="R48" s="6"/>
     </row>
     <row r="49" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I49" s="72"/>
-      <c r="J49" s="69"/>
-      <c r="K49" s="69"/>
-      <c r="L49" s="69"/>
-      <c r="M49" s="69"/>
+      <c r="I49" s="69"/>
+      <c r="J49" s="70"/>
+      <c r="K49" s="70"/>
+      <c r="L49" s="70"/>
+      <c r="M49" s="70"/>
       <c r="N49" s="9"/>
       <c r="O49" s="8">
         <v>83</v>
@@ -4674,11 +4707,11 @@
       <c r="R49" s="6"/>
     </row>
     <row r="50" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I50" s="72"/>
-      <c r="J50" s="69"/>
-      <c r="K50" s="69"/>
-      <c r="L50" s="69"/>
-      <c r="M50" s="69"/>
+      <c r="I50" s="69"/>
+      <c r="J50" s="70"/>
+      <c r="K50" s="70"/>
+      <c r="L50" s="70"/>
+      <c r="M50" s="70"/>
       <c r="N50" s="9"/>
       <c r="O50" s="8">
         <v>84</v>
@@ -4692,11 +4725,11 @@
       <c r="R50" s="6"/>
     </row>
     <row r="51" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I51" s="72"/>
-      <c r="J51" s="69"/>
-      <c r="K51" s="69"/>
-      <c r="L51" s="69"/>
-      <c r="M51" s="69"/>
+      <c r="I51" s="69"/>
+      <c r="J51" s="70"/>
+      <c r="K51" s="70"/>
+      <c r="L51" s="70"/>
+      <c r="M51" s="70"/>
       <c r="N51" s="9"/>
       <c r="O51" s="8">
         <v>85</v>
@@ -4710,11 +4743,11 @@
       <c r="R51" s="6"/>
     </row>
     <row r="52" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I52" s="72"/>
-      <c r="J52" s="69"/>
-      <c r="K52" s="69"/>
-      <c r="L52" s="69"/>
-      <c r="M52" s="69"/>
+      <c r="I52" s="69"/>
+      <c r="J52" s="70"/>
+      <c r="K52" s="70"/>
+      <c r="L52" s="70"/>
+      <c r="M52" s="70"/>
       <c r="N52" s="9"/>
       <c r="O52" s="8">
         <v>86</v>
@@ -4729,10 +4762,10 @@
     </row>
     <row r="53" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I53" s="6"/>
-      <c r="J53" s="69"/>
-      <c r="K53" s="69"/>
-      <c r="L53" s="69"/>
-      <c r="M53" s="69"/>
+      <c r="J53" s="70"/>
+      <c r="K53" s="70"/>
+      <c r="L53" s="70"/>
+      <c r="M53" s="70"/>
       <c r="N53" s="7"/>
       <c r="O53" s="8">
         <v>87</v>
@@ -4747,10 +4780,10 @@
     </row>
     <row r="54" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I54" s="6"/>
-      <c r="J54" s="69"/>
-      <c r="K54" s="69"/>
-      <c r="L54" s="69"/>
-      <c r="M54" s="69"/>
+      <c r="J54" s="70"/>
+      <c r="K54" s="70"/>
+      <c r="L54" s="70"/>
+      <c r="M54" s="70"/>
       <c r="N54" s="7"/>
       <c r="O54" s="8">
         <v>88</v>
@@ -4765,10 +4798,10 @@
     </row>
     <row r="55" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I55" s="6"/>
-      <c r="J55" s="69"/>
-      <c r="K55" s="69"/>
-      <c r="L55" s="69"/>
-      <c r="M55" s="69"/>
+      <c r="J55" s="70"/>
+      <c r="K55" s="70"/>
+      <c r="L55" s="70"/>
+      <c r="M55" s="70"/>
       <c r="N55" s="7"/>
       <c r="O55" s="8">
         <v>89</v>
@@ -4783,10 +4816,10 @@
     </row>
     <row r="56" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I56" s="6"/>
-      <c r="J56" s="69"/>
-      <c r="K56" s="69"/>
-      <c r="L56" s="69"/>
-      <c r="M56" s="69"/>
+      <c r="J56" s="70"/>
+      <c r="K56" s="70"/>
+      <c r="L56" s="70"/>
+      <c r="M56" s="70"/>
       <c r="N56" s="7"/>
       <c r="O56" s="8">
         <v>90</v>
@@ -4801,10 +4834,10 @@
     </row>
     <row r="57" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I57" s="6"/>
-      <c r="J57" s="69"/>
-      <c r="K57" s="69"/>
-      <c r="L57" s="69"/>
-      <c r="M57" s="69"/>
+      <c r="J57" s="70"/>
+      <c r="K57" s="70"/>
+      <c r="L57" s="70"/>
+      <c r="M57" s="70"/>
       <c r="N57" s="7"/>
       <c r="O57" s="8">
         <v>91</v>
@@ -4819,10 +4852,10 @@
     </row>
     <row r="58" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I58" s="6"/>
-      <c r="J58" s="69"/>
-      <c r="K58" s="69"/>
-      <c r="L58" s="69"/>
-      <c r="M58" s="69"/>
+      <c r="J58" s="70"/>
+      <c r="K58" s="70"/>
+      <c r="L58" s="70"/>
+      <c r="M58" s="70"/>
       <c r="N58" s="7"/>
       <c r="O58" s="8">
         <v>92</v>
@@ -4837,10 +4870,10 @@
     </row>
     <row r="59" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I59" s="6"/>
-      <c r="J59" s="69"/>
-      <c r="K59" s="69"/>
-      <c r="L59" s="69"/>
-      <c r="M59" s="69"/>
+      <c r="J59" s="70"/>
+      <c r="K59" s="70"/>
+      <c r="L59" s="70"/>
+      <c r="M59" s="70"/>
       <c r="N59" s="7"/>
       <c r="O59" s="8">
         <v>93</v>
@@ -4855,10 +4888,10 @@
     </row>
     <row r="60" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I60" s="6"/>
-      <c r="J60" s="69"/>
-      <c r="K60" s="69"/>
-      <c r="L60" s="69"/>
-      <c r="M60" s="69"/>
+      <c r="J60" s="70"/>
+      <c r="K60" s="70"/>
+      <c r="L60" s="70"/>
+      <c r="M60" s="70"/>
       <c r="N60" s="7"/>
       <c r="O60" s="8">
         <v>94</v>
@@ -4873,10 +4906,10 @@
     </row>
     <row r="61" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I61" s="6"/>
-      <c r="J61" s="69"/>
-      <c r="K61" s="69"/>
-      <c r="L61" s="69"/>
-      <c r="M61" s="69"/>
+      <c r="J61" s="70"/>
+      <c r="K61" s="70"/>
+      <c r="L61" s="70"/>
+      <c r="M61" s="70"/>
       <c r="N61" s="7"/>
       <c r="O61" s="8">
         <v>95</v>
@@ -4891,10 +4924,10 @@
     </row>
     <row r="62" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I62" s="6"/>
-      <c r="J62" s="69"/>
-      <c r="K62" s="69"/>
-      <c r="L62" s="69"/>
-      <c r="M62" s="69"/>
+      <c r="J62" s="70"/>
+      <c r="K62" s="70"/>
+      <c r="L62" s="70"/>
+      <c r="M62" s="70"/>
       <c r="N62" s="7"/>
       <c r="O62" s="8">
         <v>96</v>
@@ -4909,10 +4942,10 @@
     </row>
     <row r="63" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I63" s="6"/>
-      <c r="J63" s="69"/>
-      <c r="K63" s="69"/>
-      <c r="L63" s="69"/>
-      <c r="M63" s="69"/>
+      <c r="J63" s="70"/>
+      <c r="K63" s="70"/>
+      <c r="L63" s="70"/>
+      <c r="M63" s="70"/>
       <c r="N63" s="7"/>
       <c r="O63" s="8">
         <v>97</v>
@@ -4927,10 +4960,10 @@
     </row>
     <row r="64" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I64" s="6"/>
-      <c r="J64" s="69"/>
-      <c r="K64" s="69"/>
-      <c r="L64" s="69"/>
-      <c r="M64" s="69"/>
+      <c r="J64" s="70"/>
+      <c r="K64" s="70"/>
+      <c r="L64" s="70"/>
+      <c r="M64" s="70"/>
       <c r="N64" s="7"/>
       <c r="O64" s="8">
         <v>98</v>
@@ -4945,10 +4978,10 @@
     </row>
     <row r="65" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I65" s="6"/>
-      <c r="J65" s="69"/>
-      <c r="K65" s="69"/>
-      <c r="L65" s="69"/>
-      <c r="M65" s="69"/>
+      <c r="J65" s="70"/>
+      <c r="K65" s="70"/>
+      <c r="L65" s="70"/>
+      <c r="M65" s="70"/>
       <c r="N65" s="7"/>
       <c r="O65" s="8">
         <v>99</v>
@@ -4963,10 +4996,10 @@
     </row>
     <row r="66" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I66" s="6"/>
-      <c r="J66" s="69"/>
-      <c r="K66" s="69"/>
-      <c r="L66" s="69"/>
-      <c r="M66" s="69"/>
+      <c r="J66" s="70"/>
+      <c r="K66" s="70"/>
+      <c r="L66" s="70"/>
+      <c r="M66" s="70"/>
       <c r="N66" s="7"/>
       <c r="O66" s="8">
         <v>100</v>
@@ -4981,10 +5014,10 @@
     </row>
     <row r="67" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I67" s="6"/>
-      <c r="J67" s="69"/>
-      <c r="K67" s="69"/>
-      <c r="L67" s="69"/>
-      <c r="M67" s="69"/>
+      <c r="J67" s="70"/>
+      <c r="K67" s="70"/>
+      <c r="L67" s="70"/>
+      <c r="M67" s="70"/>
       <c r="N67" s="7"/>
       <c r="O67" s="8">
         <v>101</v>
@@ -4999,10 +5032,10 @@
     </row>
     <row r="68" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I68" s="6"/>
-      <c r="J68" s="69"/>
-      <c r="K68" s="69"/>
-      <c r="L68" s="69"/>
-      <c r="M68" s="69"/>
+      <c r="J68" s="70"/>
+      <c r="K68" s="70"/>
+      <c r="L68" s="70"/>
+      <c r="M68" s="70"/>
       <c r="N68" s="7"/>
       <c r="O68" s="8">
         <v>102</v>
@@ -5017,10 +5050,10 @@
     </row>
     <row r="69" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I69" s="6"/>
-      <c r="J69" s="69"/>
-      <c r="K69" s="69"/>
-      <c r="L69" s="69"/>
-      <c r="M69" s="69"/>
+      <c r="J69" s="70"/>
+      <c r="K69" s="70"/>
+      <c r="L69" s="70"/>
+      <c r="M69" s="70"/>
       <c r="N69" s="7"/>
       <c r="O69" s="8">
         <v>103</v>
@@ -5035,10 +5068,10 @@
     </row>
     <row r="70" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I70" s="6"/>
-      <c r="J70" s="69"/>
-      <c r="K70" s="69"/>
-      <c r="L70" s="69"/>
-      <c r="M70" s="69"/>
+      <c r="J70" s="70"/>
+      <c r="K70" s="70"/>
+      <c r="L70" s="70"/>
+      <c r="M70" s="70"/>
       <c r="N70" s="7"/>
       <c r="O70" s="8">
         <v>104</v>
@@ -5053,10 +5086,10 @@
     </row>
     <row r="71" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I71" s="6"/>
-      <c r="J71" s="69"/>
-      <c r="K71" s="69"/>
-      <c r="L71" s="69"/>
-      <c r="M71" s="69"/>
+      <c r="J71" s="70"/>
+      <c r="K71" s="70"/>
+      <c r="L71" s="70"/>
+      <c r="M71" s="70"/>
       <c r="N71" s="7"/>
       <c r="O71" s="8">
         <v>105</v>
@@ -5071,10 +5104,10 @@
     </row>
     <row r="72" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I72" s="6"/>
-      <c r="J72" s="69"/>
-      <c r="K72" s="69"/>
-      <c r="L72" s="69"/>
-      <c r="M72" s="69"/>
+      <c r="J72" s="70"/>
+      <c r="K72" s="70"/>
+      <c r="L72" s="70"/>
+      <c r="M72" s="70"/>
       <c r="N72" s="7"/>
       <c r="O72" s="8">
         <v>106</v>
@@ -5089,10 +5122,10 @@
     </row>
     <row r="73" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I73" s="6"/>
-      <c r="J73" s="69"/>
-      <c r="K73" s="69"/>
-      <c r="L73" s="69"/>
-      <c r="M73" s="69"/>
+      <c r="J73" s="70"/>
+      <c r="K73" s="70"/>
+      <c r="L73" s="70"/>
+      <c r="M73" s="70"/>
       <c r="N73" s="7"/>
       <c r="O73" s="8">
         <v>107</v>
@@ -5107,10 +5140,10 @@
     </row>
     <row r="74" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I74" s="6"/>
-      <c r="J74" s="69"/>
-      <c r="K74" s="69"/>
-      <c r="L74" s="69"/>
-      <c r="M74" s="69"/>
+      <c r="J74" s="70"/>
+      <c r="K74" s="70"/>
+      <c r="L74" s="70"/>
+      <c r="M74" s="70"/>
       <c r="N74" s="7"/>
       <c r="O74" s="8">
         <v>108</v>
@@ -5125,10 +5158,10 @@
     </row>
     <row r="75" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I75" s="6"/>
-      <c r="J75" s="69"/>
-      <c r="K75" s="69"/>
-      <c r="L75" s="69"/>
-      <c r="M75" s="69"/>
+      <c r="J75" s="70"/>
+      <c r="K75" s="70"/>
+      <c r="L75" s="70"/>
+      <c r="M75" s="70"/>
       <c r="N75" s="7"/>
       <c r="O75" s="8">
         <v>109</v>
@@ -5143,10 +5176,10 @@
     </row>
     <row r="76" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I76" s="6"/>
-      <c r="J76" s="69"/>
-      <c r="K76" s="69"/>
-      <c r="L76" s="69"/>
-      <c r="M76" s="69"/>
+      <c r="J76" s="70"/>
+      <c r="K76" s="70"/>
+      <c r="L76" s="70"/>
+      <c r="M76" s="70"/>
       <c r="N76" s="7"/>
       <c r="O76" s="8">
         <v>110</v>
@@ -5161,10 +5194,10 @@
     </row>
     <row r="77" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I77" s="6"/>
-      <c r="J77" s="69"/>
-      <c r="K77" s="69"/>
-      <c r="L77" s="69"/>
-      <c r="M77" s="69"/>
+      <c r="J77" s="70"/>
+      <c r="K77" s="70"/>
+      <c r="L77" s="70"/>
+      <c r="M77" s="70"/>
       <c r="N77" s="7"/>
       <c r="O77" s="8">
         <v>111</v>
@@ -5179,10 +5212,10 @@
     </row>
     <row r="78" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I78" s="6"/>
-      <c r="J78" s="69"/>
-      <c r="K78" s="69"/>
-      <c r="L78" s="69"/>
-      <c r="M78" s="69"/>
+      <c r="J78" s="70"/>
+      <c r="K78" s="70"/>
+      <c r="L78" s="70"/>
+      <c r="M78" s="70"/>
       <c r="N78" s="7"/>
       <c r="O78" s="8">
         <v>112</v>
@@ -5197,10 +5230,10 @@
     </row>
     <row r="79" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I79" s="6"/>
-      <c r="J79" s="69"/>
-      <c r="K79" s="69"/>
-      <c r="L79" s="69"/>
-      <c r="M79" s="69"/>
+      <c r="J79" s="70"/>
+      <c r="K79" s="70"/>
+      <c r="L79" s="70"/>
+      <c r="M79" s="70"/>
       <c r="N79" s="7"/>
       <c r="O79" s="8">
         <v>113</v>
@@ -5215,10 +5248,10 @@
     </row>
     <row r="80" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I80" s="6"/>
-      <c r="J80" s="69"/>
-      <c r="K80" s="69"/>
-      <c r="L80" s="69"/>
-      <c r="M80" s="69"/>
+      <c r="J80" s="70"/>
+      <c r="K80" s="70"/>
+      <c r="L80" s="70"/>
+      <c r="M80" s="70"/>
       <c r="N80" s="7"/>
       <c r="O80" s="8">
         <v>114</v>
@@ -5233,10 +5266,10 @@
     </row>
     <row r="81" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I81" s="6"/>
-      <c r="J81" s="69"/>
-      <c r="K81" s="69"/>
-      <c r="L81" s="69"/>
-      <c r="M81" s="69"/>
+      <c r="J81" s="70"/>
+      <c r="K81" s="70"/>
+      <c r="L81" s="70"/>
+      <c r="M81" s="70"/>
       <c r="N81" s="7"/>
       <c r="O81" s="8">
         <v>115</v>
@@ -5251,10 +5284,10 @@
     </row>
     <row r="82" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I82" s="6"/>
-      <c r="J82" s="69"/>
-      <c r="K82" s="69"/>
-      <c r="L82" s="69"/>
-      <c r="M82" s="69"/>
+      <c r="J82" s="70"/>
+      <c r="K82" s="70"/>
+      <c r="L82" s="70"/>
+      <c r="M82" s="70"/>
       <c r="N82" s="7"/>
       <c r="O82" s="8">
         <v>116</v>
@@ -5269,10 +5302,10 @@
     </row>
     <row r="83" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I83" s="6"/>
-      <c r="J83" s="69"/>
-      <c r="K83" s="69"/>
-      <c r="L83" s="69"/>
-      <c r="M83" s="69"/>
+      <c r="J83" s="70"/>
+      <c r="K83" s="70"/>
+      <c r="L83" s="70"/>
+      <c r="M83" s="70"/>
       <c r="N83" s="7"/>
       <c r="O83" s="8">
         <v>117</v>
@@ -5287,10 +5320,10 @@
     </row>
     <row r="84" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I84" s="6"/>
-      <c r="J84" s="69"/>
-      <c r="K84" s="69"/>
-      <c r="L84" s="69"/>
-      <c r="M84" s="69"/>
+      <c r="J84" s="70"/>
+      <c r="K84" s="70"/>
+      <c r="L84" s="70"/>
+      <c r="M84" s="70"/>
       <c r="N84" s="7"/>
       <c r="O84" s="8">
         <v>118</v>
@@ -5305,10 +5338,10 @@
     </row>
     <row r="85" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I85" s="6"/>
-      <c r="J85" s="69"/>
-      <c r="K85" s="69"/>
-      <c r="L85" s="69"/>
-      <c r="M85" s="69"/>
+      <c r="J85" s="70"/>
+      <c r="K85" s="70"/>
+      <c r="L85" s="70"/>
+      <c r="M85" s="70"/>
       <c r="N85" s="7"/>
       <c r="O85" s="8">
         <v>119</v>
@@ -5323,10 +5356,10 @@
     </row>
     <row r="86" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I86" s="6"/>
-      <c r="J86" s="69"/>
-      <c r="K86" s="69"/>
-      <c r="L86" s="69"/>
-      <c r="M86" s="69"/>
+      <c r="J86" s="70"/>
+      <c r="K86" s="70"/>
+      <c r="L86" s="70"/>
+      <c r="M86" s="70"/>
       <c r="N86" s="7"/>
       <c r="O86" s="8">
         <v>120</v>
@@ -5341,10 +5374,10 @@
     </row>
     <row r="87" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I87" s="6"/>
-      <c r="J87" s="69"/>
-      <c r="K87" s="69"/>
-      <c r="L87" s="69"/>
-      <c r="M87" s="69"/>
+      <c r="J87" s="70"/>
+      <c r="K87" s="70"/>
+      <c r="L87" s="70"/>
+      <c r="M87" s="70"/>
       <c r="N87" s="7"/>
       <c r="O87" s="8">
         <v>121</v>
@@ -5359,10 +5392,10 @@
     </row>
     <row r="88" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I88" s="6"/>
-      <c r="J88" s="69"/>
-      <c r="K88" s="69"/>
-      <c r="L88" s="69"/>
-      <c r="M88" s="69"/>
+      <c r="J88" s="70"/>
+      <c r="K88" s="70"/>
+      <c r="L88" s="70"/>
+      <c r="M88" s="70"/>
       <c r="N88" s="7"/>
       <c r="O88" s="8">
         <v>122</v>
@@ -5377,10 +5410,10 @@
     </row>
     <row r="89" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I89" s="6"/>
-      <c r="J89" s="69"/>
-      <c r="K89" s="69"/>
-      <c r="L89" s="69"/>
-      <c r="M89" s="69"/>
+      <c r="J89" s="70"/>
+      <c r="K89" s="70"/>
+      <c r="L89" s="70"/>
+      <c r="M89" s="70"/>
       <c r="N89" s="7"/>
       <c r="O89" s="8">
         <v>123</v>
@@ -5395,10 +5428,10 @@
     </row>
     <row r="90" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I90" s="6"/>
-      <c r="J90" s="69"/>
-      <c r="K90" s="69"/>
-      <c r="L90" s="69"/>
-      <c r="M90" s="69"/>
+      <c r="J90" s="70"/>
+      <c r="K90" s="70"/>
+      <c r="L90" s="70"/>
+      <c r="M90" s="70"/>
       <c r="N90" s="7"/>
       <c r="O90" s="8">
         <v>124</v>
@@ -5413,10 +5446,10 @@
     </row>
     <row r="91" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I91" s="6"/>
-      <c r="J91" s="69"/>
-      <c r="K91" s="69"/>
-      <c r="L91" s="69"/>
-      <c r="M91" s="69"/>
+      <c r="J91" s="70"/>
+      <c r="K91" s="70"/>
+      <c r="L91" s="70"/>
+      <c r="M91" s="70"/>
       <c r="N91" s="7"/>
       <c r="O91" s="8">
         <v>125</v>
@@ -5431,10 +5464,10 @@
     </row>
     <row r="92" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I92" s="6"/>
-      <c r="J92" s="69"/>
-      <c r="K92" s="69"/>
-      <c r="L92" s="69"/>
-      <c r="M92" s="69"/>
+      <c r="J92" s="70"/>
+      <c r="K92" s="70"/>
+      <c r="L92" s="70"/>
+      <c r="M92" s="70"/>
       <c r="N92" s="7"/>
       <c r="O92" s="8">
         <v>126</v>
@@ -5449,10 +5482,10 @@
     </row>
     <row r="93" spans="9:18" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I93" s="6"/>
-      <c r="J93" s="69"/>
-      <c r="K93" s="69"/>
-      <c r="L93" s="69"/>
-      <c r="M93" s="69"/>
+      <c r="J93" s="70"/>
+      <c r="K93" s="70"/>
+      <c r="L93" s="70"/>
+      <c r="M93" s="70"/>
       <c r="N93" s="7"/>
       <c r="O93" s="8">
         <v>127</v>
@@ -7645,31 +7678,47 @@
     </row>
   </sheetData>
   <mergeCells count="80">
-    <mergeCell ref="J15:M15"/>
-    <mergeCell ref="J16:M16"/>
-    <mergeCell ref="J17:M17"/>
-    <mergeCell ref="J18:M18"/>
-    <mergeCell ref="J19:M19"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="J27:M27"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="J28:M28"/>
-    <mergeCell ref="J29:M29"/>
-    <mergeCell ref="J30:M30"/>
-    <mergeCell ref="J31:M31"/>
-    <mergeCell ref="J32:M32"/>
-    <mergeCell ref="J33:M33"/>
-    <mergeCell ref="J34:M34"/>
-    <mergeCell ref="J35:M35"/>
-    <mergeCell ref="J36:M36"/>
-    <mergeCell ref="J37:M37"/>
-    <mergeCell ref="J38:M38"/>
-    <mergeCell ref="J39:M39"/>
+    <mergeCell ref="J93:M93"/>
+    <mergeCell ref="J88:M88"/>
+    <mergeCell ref="J89:M89"/>
+    <mergeCell ref="J90:M90"/>
+    <mergeCell ref="J91:M91"/>
+    <mergeCell ref="J92:M92"/>
+    <mergeCell ref="J83:M83"/>
+    <mergeCell ref="J84:M84"/>
+    <mergeCell ref="J85:M85"/>
+    <mergeCell ref="J86:M86"/>
+    <mergeCell ref="J87:M87"/>
+    <mergeCell ref="J78:M78"/>
+    <mergeCell ref="J79:M79"/>
+    <mergeCell ref="J80:M80"/>
+    <mergeCell ref="J81:M81"/>
+    <mergeCell ref="J82:M82"/>
+    <mergeCell ref="J73:M73"/>
+    <mergeCell ref="J74:M74"/>
+    <mergeCell ref="J75:M75"/>
+    <mergeCell ref="J76:M76"/>
+    <mergeCell ref="J77:M77"/>
+    <mergeCell ref="J68:M68"/>
+    <mergeCell ref="J69:M69"/>
+    <mergeCell ref="J70:M70"/>
+    <mergeCell ref="J71:M71"/>
+    <mergeCell ref="J72:M72"/>
+    <mergeCell ref="J63:M63"/>
+    <mergeCell ref="J64:M64"/>
+    <mergeCell ref="J65:M65"/>
+    <mergeCell ref="J66:M66"/>
+    <mergeCell ref="J67:M67"/>
+    <mergeCell ref="J58:M58"/>
+    <mergeCell ref="J59:M59"/>
+    <mergeCell ref="J60:M60"/>
+    <mergeCell ref="J61:M61"/>
+    <mergeCell ref="J62:M62"/>
+    <mergeCell ref="J53:M53"/>
+    <mergeCell ref="J54:M54"/>
+    <mergeCell ref="J55:M55"/>
+    <mergeCell ref="J56:M56"/>
+    <mergeCell ref="J57:M57"/>
     <mergeCell ref="J40:M40"/>
     <mergeCell ref="J41:M41"/>
     <mergeCell ref="J42:M42"/>
@@ -7684,47 +7733,31 @@
     <mergeCell ref="J50:M50"/>
     <mergeCell ref="J51:M51"/>
     <mergeCell ref="J52:M52"/>
-    <mergeCell ref="J53:M53"/>
-    <mergeCell ref="J54:M54"/>
-    <mergeCell ref="J55:M55"/>
-    <mergeCell ref="J56:M56"/>
-    <mergeCell ref="J57:M57"/>
-    <mergeCell ref="J58:M58"/>
-    <mergeCell ref="J59:M59"/>
-    <mergeCell ref="J60:M60"/>
-    <mergeCell ref="J61:M61"/>
-    <mergeCell ref="J62:M62"/>
-    <mergeCell ref="J63:M63"/>
-    <mergeCell ref="J64:M64"/>
-    <mergeCell ref="J65:M65"/>
-    <mergeCell ref="J66:M66"/>
-    <mergeCell ref="J67:M67"/>
-    <mergeCell ref="J68:M68"/>
-    <mergeCell ref="J69:M69"/>
-    <mergeCell ref="J70:M70"/>
-    <mergeCell ref="J71:M71"/>
-    <mergeCell ref="J72:M72"/>
-    <mergeCell ref="J73:M73"/>
-    <mergeCell ref="J74:M74"/>
-    <mergeCell ref="J75:M75"/>
-    <mergeCell ref="J76:M76"/>
-    <mergeCell ref="J77:M77"/>
-    <mergeCell ref="J78:M78"/>
-    <mergeCell ref="J79:M79"/>
-    <mergeCell ref="J80:M80"/>
-    <mergeCell ref="J81:M81"/>
-    <mergeCell ref="J82:M82"/>
-    <mergeCell ref="J83:M83"/>
-    <mergeCell ref="J84:M84"/>
-    <mergeCell ref="J85:M85"/>
-    <mergeCell ref="J86:M86"/>
-    <mergeCell ref="J87:M87"/>
-    <mergeCell ref="J93:M93"/>
-    <mergeCell ref="J88:M88"/>
-    <mergeCell ref="J89:M89"/>
-    <mergeCell ref="J90:M90"/>
-    <mergeCell ref="J91:M91"/>
-    <mergeCell ref="J92:M92"/>
+    <mergeCell ref="J35:M35"/>
+    <mergeCell ref="J36:M36"/>
+    <mergeCell ref="J37:M37"/>
+    <mergeCell ref="J38:M38"/>
+    <mergeCell ref="J39:M39"/>
+    <mergeCell ref="J30:M30"/>
+    <mergeCell ref="J31:M31"/>
+    <mergeCell ref="J32:M32"/>
+    <mergeCell ref="J33:M33"/>
+    <mergeCell ref="J34:M34"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="J27:M27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="J28:M28"/>
+    <mergeCell ref="J29:M29"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="J15:M15"/>
+    <mergeCell ref="J16:M16"/>
+    <mergeCell ref="J17:M17"/>
+    <mergeCell ref="J18:M18"/>
+    <mergeCell ref="J19:M19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7824,1125 +7857,1125 @@
       <c r="U1" s="20"/>
     </row>
     <row r="2" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="42"/>
-      <c r="B2" s="42" t="s">
+      <c r="A2" s="41"/>
+      <c r="B2" s="41" t="s">
         <v>553</v>
       </c>
-      <c r="C2" s="42" t="s">
+      <c r="C2" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="43" t="s">
+      <c r="D2" s="42" t="s">
         <v>554</v>
       </c>
-      <c r="E2" s="42" t="s">
+      <c r="E2" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
-      <c r="N2" s="42"/>
-      <c r="O2" s="42" t="s">
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41" t="s">
         <v>556</v>
       </c>
-      <c r="P2" s="42" t="s">
+      <c r="P2" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q2" s="44" t="s">
+      <c r="Q2" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R2" s="42" t="s">
+      <c r="R2" s="41" t="s">
         <v>558</v>
       </c>
-      <c r="S2" s="42" t="s">
+      <c r="S2" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="41" t="s">
         <v>513</v>
       </c>
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="41" t="s">
         <v>559</v>
       </c>
-      <c r="C3" s="42" t="s">
+      <c r="C3" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="42" t="s">
         <v>560</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="42"/>
-      <c r="J3" s="42"/>
-      <c r="K3" s="42"/>
-      <c r="L3" s="42"/>
-      <c r="M3" s="42"/>
-      <c r="N3" s="42"/>
-      <c r="O3" s="42" t="s">
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="41"/>
+      <c r="J3" s="41"/>
+      <c r="K3" s="41"/>
+      <c r="L3" s="41"/>
+      <c r="M3" s="41"/>
+      <c r="N3" s="41"/>
+      <c r="O3" s="41" t="s">
         <v>561</v>
       </c>
-      <c r="P3" s="42" t="s">
+      <c r="P3" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q3" s="44" t="s">
+      <c r="Q3" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R3" s="42" t="s">
+      <c r="R3" s="41" t="s">
         <v>562</v>
       </c>
-      <c r="S3" s="42" t="s">
+      <c r="S3" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="41" t="s">
         <v>563</v>
       </c>
-      <c r="B4" s="42" t="s">
+      <c r="B4" s="41" t="s">
         <v>564</v>
       </c>
-      <c r="C4" s="42" t="s">
+      <c r="C4" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="43" t="s">
+      <c r="D4" s="42" t="s">
         <v>565</v>
       </c>
-      <c r="E4" s="42" t="s">
+      <c r="E4" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="42"/>
-      <c r="I4" s="42"/>
-      <c r="J4" s="42"/>
-      <c r="K4" s="42"/>
-      <c r="L4" s="42"/>
-      <c r="M4" s="42"/>
-      <c r="N4" s="42"/>
-      <c r="O4" s="42" t="s">
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="41"/>
+      <c r="M4" s="41"/>
+      <c r="N4" s="41"/>
+      <c r="O4" s="41" t="s">
         <v>561</v>
       </c>
-      <c r="P4" s="42" t="s">
+      <c r="P4" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q4" s="44" t="s">
+      <c r="Q4" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R4" s="42" t="s">
+      <c r="R4" s="41" t="s">
         <v>566</v>
       </c>
-      <c r="S4" s="42" t="s">
+      <c r="S4" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="41" t="s">
         <v>567</v>
       </c>
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="41" t="s">
         <v>568</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="43" t="s">
+      <c r="D5" s="42" t="s">
         <v>569</v>
       </c>
-      <c r="E5" s="42" t="s">
+      <c r="E5" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
-      <c r="K5" s="42"/>
-      <c r="L5" s="42"/>
-      <c r="M5" s="42"/>
-      <c r="N5" s="42"/>
-      <c r="O5" s="42" t="s">
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+      <c r="M5" s="41"/>
+      <c r="N5" s="41"/>
+      <c r="O5" s="41" t="s">
         <v>561</v>
       </c>
-      <c r="P5" s="42" t="s">
+      <c r="P5" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q5" s="44" t="s">
+      <c r="Q5" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R5" s="42" t="s">
+      <c r="R5" s="41" t="s">
         <v>570</v>
       </c>
-      <c r="S5" s="42" t="s">
+      <c r="S5" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A6" s="42" t="s">
+      <c r="A6" s="41" t="s">
         <v>571</v>
       </c>
-      <c r="B6" s="42"/>
-      <c r="C6" s="42" t="s">
+      <c r="B6" s="41"/>
+      <c r="C6" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="43" t="s">
+      <c r="D6" s="42" t="s">
         <v>572</v>
       </c>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="42"/>
-      <c r="I6" s="42"/>
-      <c r="J6" s="42"/>
-      <c r="K6" s="42"/>
-      <c r="L6" s="42"/>
-      <c r="M6" s="42"/>
-      <c r="N6" s="42"/>
-      <c r="O6" s="42" t="s">
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="41"/>
+      <c r="L6" s="41"/>
+      <c r="M6" s="41"/>
+      <c r="N6" s="41"/>
+      <c r="O6" s="41" t="s">
         <v>573</v>
       </c>
-      <c r="P6" s="42" t="s">
+      <c r="P6" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q6" s="44" t="s">
+      <c r="Q6" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R6" s="45" t="s">
+      <c r="R6" s="44" t="s">
         <v>574</v>
       </c>
-      <c r="S6" s="42" t="s">
+      <c r="S6" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A7" s="42" t="s">
+      <c r="A7" s="41" t="s">
         <v>571</v>
       </c>
-      <c r="B7" s="42" t="s">
+      <c r="B7" s="41" t="s">
         <v>513</v>
       </c>
-      <c r="C7" s="42" t="s">
+      <c r="C7" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="42" t="s">
         <v>575</v>
       </c>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="42"/>
-      <c r="H7" s="42"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="42"/>
-      <c r="K7" s="42"/>
-      <c r="L7" s="42"/>
-      <c r="M7" s="42"/>
-      <c r="N7" s="42"/>
-      <c r="O7" s="42" t="s">
+      <c r="F7" s="41"/>
+      <c r="G7" s="41"/>
+      <c r="H7" s="41"/>
+      <c r="I7" s="41"/>
+      <c r="J7" s="41"/>
+      <c r="K7" s="41"/>
+      <c r="L7" s="41"/>
+      <c r="M7" s="41"/>
+      <c r="N7" s="41"/>
+      <c r="O7" s="41" t="s">
         <v>576</v>
       </c>
-      <c r="P7" s="42" t="s">
+      <c r="P7" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q7" s="44" t="s">
+      <c r="Q7" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R7" s="42" t="s">
+      <c r="R7" s="41" t="s">
         <v>577</v>
       </c>
-      <c r="S7" s="42" t="s">
+      <c r="S7" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A8" s="42" t="s">
+      <c r="A8" s="41" t="s">
         <v>571</v>
       </c>
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="41" t="s">
         <v>513</v>
       </c>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="43" t="s">
+      <c r="D8" s="42" t="s">
         <v>578</v>
       </c>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F8" s="42"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="42"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="42"/>
-      <c r="K8" s="42"/>
-      <c r="L8" s="42"/>
-      <c r="M8" s="42"/>
-      <c r="N8" s="42"/>
-      <c r="O8" s="42" t="s">
+      <c r="F8" s="41"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="41"/>
+      <c r="I8" s="41"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="41"/>
+      <c r="L8" s="41"/>
+      <c r="M8" s="41"/>
+      <c r="N8" s="41"/>
+      <c r="O8" s="41" t="s">
         <v>576</v>
       </c>
-      <c r="P8" s="42" t="s">
+      <c r="P8" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q8" s="44" t="s">
+      <c r="Q8" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R8" s="42" t="s">
+      <c r="R8" s="41" t="s">
         <v>579</v>
       </c>
-      <c r="S8" s="42" t="s">
+      <c r="S8" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A9" s="42" t="s">
+      <c r="A9" s="41" t="s">
         <v>571</v>
       </c>
-      <c r="B9" s="42" t="s">
+      <c r="B9" s="41" t="s">
         <v>580</v>
       </c>
-      <c r="C9" s="42" t="s">
+      <c r="C9" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="43" t="s">
+      <c r="D9" s="42" t="s">
         <v>578</v>
       </c>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="42"/>
-      <c r="H9" s="42"/>
-      <c r="I9" s="42"/>
-      <c r="J9" s="42"/>
-      <c r="K9" s="42"/>
-      <c r="L9" s="42"/>
-      <c r="M9" s="42"/>
-      <c r="N9" s="42"/>
-      <c r="O9" s="42" t="s">
+      <c r="F9" s="41"/>
+      <c r="G9" s="41"/>
+      <c r="H9" s="41"/>
+      <c r="I9" s="41"/>
+      <c r="J9" s="41"/>
+      <c r="K9" s="41"/>
+      <c r="L9" s="41"/>
+      <c r="M9" s="41"/>
+      <c r="N9" s="41"/>
+      <c r="O9" s="41" t="s">
         <v>576</v>
       </c>
-      <c r="P9" s="42" t="s">
+      <c r="P9" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q9" s="44" t="s">
+      <c r="Q9" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R9" s="42" t="s">
+      <c r="R9" s="41" t="s">
         <v>581</v>
       </c>
-      <c r="S9" s="42" t="s">
+      <c r="S9" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A10" s="42" t="s">
+      <c r="A10" s="41" t="s">
         <v>571</v>
       </c>
-      <c r="B10" s="42" t="s">
+      <c r="B10" s="41" t="s">
         <v>582</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="43" t="s">
+      <c r="D10" s="42" t="s">
         <v>583</v>
       </c>
-      <c r="E10" s="42" t="s">
+      <c r="E10" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F10" s="42"/>
-      <c r="G10" s="42"/>
-      <c r="H10" s="42"/>
-      <c r="I10" s="42"/>
-      <c r="J10" s="42"/>
-      <c r="K10" s="42"/>
-      <c r="L10" s="42"/>
-      <c r="M10" s="42"/>
-      <c r="N10" s="42"/>
-      <c r="O10" s="42" t="s">
+      <c r="F10" s="41"/>
+      <c r="G10" s="41"/>
+      <c r="H10" s="41"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="41"/>
+      <c r="K10" s="41"/>
+      <c r="L10" s="41"/>
+      <c r="M10" s="41"/>
+      <c r="N10" s="41"/>
+      <c r="O10" s="41" t="s">
         <v>576</v>
       </c>
-      <c r="P10" s="42" t="s">
+      <c r="P10" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q10" s="44" t="s">
+      <c r="Q10" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R10" s="42" t="s">
+      <c r="R10" s="41" t="s">
         <v>584</v>
       </c>
-      <c r="S10" s="42" t="s">
+      <c r="S10" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="41" t="s">
         <v>571</v>
       </c>
-      <c r="B11" s="42" t="s">
+      <c r="B11" s="41" t="s">
         <v>585</v>
       </c>
-      <c r="C11" s="42" t="s">
+      <c r="C11" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="43" t="s">
+      <c r="D11" s="42" t="s">
         <v>586</v>
       </c>
-      <c r="E11" s="42" t="s">
+      <c r="E11" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
-      <c r="K11" s="42"/>
-      <c r="L11" s="42"/>
-      <c r="M11" s="42"/>
-      <c r="N11" s="42"/>
-      <c r="O11" s="42" t="s">
+      <c r="F11" s="41"/>
+      <c r="G11" s="41"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="41"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="41"/>
+      <c r="M11" s="41"/>
+      <c r="N11" s="41"/>
+      <c r="O11" s="41" t="s">
         <v>576</v>
       </c>
-      <c r="P11" s="42" t="s">
+      <c r="P11" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q11" s="44" t="s">
+      <c r="Q11" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R11" s="42" t="s">
+      <c r="R11" s="41" t="s">
         <v>587</v>
       </c>
-      <c r="S11" s="42" t="s">
+      <c r="S11" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A12" s="42" t="s">
+      <c r="A12" s="41" t="s">
         <v>588</v>
       </c>
-      <c r="B12" s="42" t="s">
+      <c r="B12" s="41" t="s">
         <v>589</v>
       </c>
-      <c r="C12" s="42" t="s">
+      <c r="C12" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="46"/>
-      <c r="E12" s="42" t="s">
+      <c r="D12" s="45"/>
+      <c r="E12" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="42"/>
-      <c r="J12" s="42"/>
-      <c r="K12" s="42"/>
-      <c r="L12" s="42"/>
-      <c r="M12" s="42"/>
-      <c r="N12" s="42"/>
-      <c r="O12" s="42" t="s">
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
+      <c r="K12" s="41"/>
+      <c r="L12" s="41"/>
+      <c r="M12" s="41"/>
+      <c r="N12" s="41"/>
+      <c r="O12" s="41" t="s">
         <v>590</v>
       </c>
-      <c r="P12" s="42" t="s">
+      <c r="P12" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q12" s="44" t="s">
+      <c r="Q12" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R12" s="45" t="s">
+      <c r="R12" s="44" t="s">
         <v>591</v>
       </c>
-      <c r="S12" s="42" t="s">
+      <c r="S12" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A13" s="42" t="s">
+      <c r="A13" s="41" t="s">
         <v>588</v>
       </c>
-      <c r="B13" s="42" t="s">
+      <c r="B13" s="41" t="s">
         <v>592</v>
       </c>
-      <c r="C13" s="42" t="s">
+      <c r="C13" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="43" t="s">
+      <c r="D13" s="42" t="s">
         <v>513</v>
       </c>
-      <c r="E13" s="42" t="s">
+      <c r="E13" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="42"/>
-      <c r="J13" s="42"/>
-      <c r="K13" s="42"/>
-      <c r="L13" s="42"/>
-      <c r="M13" s="42"/>
-      <c r="N13" s="42"/>
-      <c r="O13" s="42" t="s">
+      <c r="F13" s="41"/>
+      <c r="G13" s="41"/>
+      <c r="H13" s="41"/>
+      <c r="I13" s="41"/>
+      <c r="J13" s="41"/>
+      <c r="K13" s="41"/>
+      <c r="L13" s="41"/>
+      <c r="M13" s="41"/>
+      <c r="N13" s="41"/>
+      <c r="O13" s="41" t="s">
         <v>593</v>
       </c>
-      <c r="P13" s="42" t="s">
+      <c r="P13" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q13" s="44" t="s">
+      <c r="Q13" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R13" s="42" t="s">
+      <c r="R13" s="41" t="s">
         <v>594</v>
       </c>
-      <c r="S13" s="42" t="s">
+      <c r="S13" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A14" s="42" t="s">
+      <c r="A14" s="41" t="s">
         <v>588</v>
       </c>
-      <c r="B14" s="42" t="s">
+      <c r="B14" s="41" t="s">
         <v>595</v>
       </c>
-      <c r="C14" s="42" t="s">
+      <c r="C14" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="43" t="s">
+      <c r="D14" s="42" t="s">
         <v>596</v>
       </c>
-      <c r="E14" s="42" t="s">
+      <c r="E14" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F14" s="42"/>
-      <c r="G14" s="42"/>
-      <c r="H14" s="42"/>
-      <c r="I14" s="42"/>
-      <c r="J14" s="42"/>
-      <c r="K14" s="42"/>
-      <c r="L14" s="42"/>
-      <c r="M14" s="42"/>
-      <c r="N14" s="42"/>
-      <c r="O14" s="42" t="s">
+      <c r="F14" s="41"/>
+      <c r="G14" s="41"/>
+      <c r="H14" s="41"/>
+      <c r="I14" s="41"/>
+      <c r="J14" s="41"/>
+      <c r="K14" s="41"/>
+      <c r="L14" s="41"/>
+      <c r="M14" s="41"/>
+      <c r="N14" s="41"/>
+      <c r="O14" s="41" t="s">
         <v>593</v>
       </c>
-      <c r="P14" s="42" t="s">
+      <c r="P14" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q14" s="44" t="s">
+      <c r="Q14" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R14" s="42" t="s">
+      <c r="R14" s="41" t="s">
         <v>597</v>
       </c>
-      <c r="S14" s="42" t="s">
+      <c r="S14" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A15" s="42" t="s">
+      <c r="A15" s="41" t="s">
         <v>588</v>
       </c>
-      <c r="B15" s="42" t="s">
+      <c r="B15" s="41" t="s">
         <v>598</v>
       </c>
-      <c r="C15" s="42" t="s">
+      <c r="C15" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="43" t="s">
+      <c r="D15" s="42" t="s">
         <v>599</v>
       </c>
-      <c r="E15" s="42" t="s">
+      <c r="E15" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="42"/>
-      <c r="J15" s="42"/>
-      <c r="K15" s="42"/>
-      <c r="L15" s="42"/>
-      <c r="M15" s="42"/>
-      <c r="N15" s="42"/>
-      <c r="O15" s="42" t="s">
+      <c r="F15" s="41"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="41"/>
+      <c r="L15" s="41"/>
+      <c r="M15" s="41"/>
+      <c r="N15" s="41"/>
+      <c r="O15" s="41" t="s">
         <v>593</v>
       </c>
-      <c r="P15" s="42" t="s">
+      <c r="P15" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q15" s="44" t="s">
+      <c r="Q15" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R15" s="42" t="s">
+      <c r="R15" s="41" t="s">
         <v>600</v>
       </c>
-      <c r="S15" s="42" t="s">
+      <c r="S15" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A16" s="42" t="s">
+      <c r="A16" s="41" t="s">
         <v>588</v>
       </c>
-      <c r="B16" s="42" t="s">
+      <c r="B16" s="41" t="s">
         <v>601</v>
       </c>
-      <c r="C16" s="42" t="s">
+      <c r="C16" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="43" t="s">
+      <c r="D16" s="42" t="s">
         <v>602</v>
       </c>
-      <c r="E16" s="42" t="s">
+      <c r="E16" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F16" s="42"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="42"/>
-      <c r="I16" s="42"/>
-      <c r="J16" s="42"/>
-      <c r="K16" s="42"/>
-      <c r="L16" s="42"/>
-      <c r="M16" s="42"/>
-      <c r="N16" s="42"/>
-      <c r="O16" s="42" t="s">
+      <c r="F16" s="41"/>
+      <c r="G16" s="41"/>
+      <c r="H16" s="41"/>
+      <c r="I16" s="41"/>
+      <c r="J16" s="41"/>
+      <c r="K16" s="41"/>
+      <c r="L16" s="41"/>
+      <c r="M16" s="41"/>
+      <c r="N16" s="41"/>
+      <c r="O16" s="41" t="s">
         <v>593</v>
       </c>
-      <c r="P16" s="42" t="s">
+      <c r="P16" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q16" s="44" t="s">
+      <c r="Q16" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R16" s="42" t="s">
+      <c r="R16" s="41" t="s">
         <v>603</v>
       </c>
-      <c r="S16" s="42" t="s">
+      <c r="S16" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="41" t="s">
         <v>604</v>
       </c>
-      <c r="B17" s="42" t="s">
+      <c r="B17" s="41" t="s">
         <v>605</v>
       </c>
-      <c r="C17" s="42"/>
-      <c r="D17" s="43" t="s">
+      <c r="C17" s="41"/>
+      <c r="D17" s="42" t="s">
         <v>606</v>
       </c>
-      <c r="E17" s="42" t="s">
+      <c r="E17" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F17" s="42"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="42"/>
-      <c r="I17" s="42"/>
-      <c r="J17" s="42"/>
-      <c r="K17" s="42"/>
-      <c r="L17" s="42"/>
-      <c r="M17" s="42"/>
-      <c r="N17" s="42"/>
-      <c r="O17" s="42" t="s">
+      <c r="F17" s="41"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="41"/>
+      <c r="K17" s="41"/>
+      <c r="L17" s="41"/>
+      <c r="M17" s="41"/>
+      <c r="N17" s="41"/>
+      <c r="O17" s="41" t="s">
         <v>478</v>
       </c>
-      <c r="P17" s="42" t="s">
+      <c r="P17" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q17" s="44" t="s">
+      <c r="Q17" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R17" s="42" t="s">
+      <c r="R17" s="41" t="s">
         <v>481</v>
       </c>
-      <c r="S17" s="42" t="s">
+      <c r="S17" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A18" s="42" t="s">
+      <c r="A18" s="41" t="s">
         <v>604</v>
       </c>
-      <c r="B18" s="42" t="s">
+      <c r="B18" s="41" t="s">
         <v>607</v>
       </c>
-      <c r="C18" s="42" t="s">
+      <c r="C18" s="41" t="s">
         <v>513</v>
       </c>
-      <c r="D18" s="43" t="s">
+      <c r="D18" s="42" t="s">
         <v>608</v>
       </c>
-      <c r="E18" s="42" t="s">
+      <c r="E18" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F18" s="42"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="42"/>
-      <c r="J18" s="42"/>
-      <c r="K18" s="42"/>
-      <c r="L18" s="42"/>
-      <c r="M18" s="42"/>
-      <c r="N18" s="42"/>
-      <c r="O18" s="42" t="s">
+      <c r="F18" s="41"/>
+      <c r="G18" s="41"/>
+      <c r="H18" s="41"/>
+      <c r="I18" s="41"/>
+      <c r="J18" s="41"/>
+      <c r="K18" s="41"/>
+      <c r="L18" s="41"/>
+      <c r="M18" s="41"/>
+      <c r="N18" s="41"/>
+      <c r="O18" s="41" t="s">
         <v>609</v>
       </c>
-      <c r="P18" s="42" t="s">
+      <c r="P18" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q18" s="44" t="s">
+      <c r="Q18" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R18" s="42" t="s">
+      <c r="R18" s="41" t="s">
         <v>484</v>
       </c>
-      <c r="S18" s="42" t="s">
+      <c r="S18" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A19" s="42" t="s">
+      <c r="A19" s="41" t="s">
         <v>604</v>
       </c>
-      <c r="B19" s="42" t="s">
+      <c r="B19" s="41" t="s">
         <v>610</v>
       </c>
-      <c r="C19" s="42" t="s">
+      <c r="C19" s="41" t="s">
         <v>611</v>
       </c>
-      <c r="D19" s="43" t="s">
+      <c r="D19" s="42" t="s">
         <v>612</v>
       </c>
-      <c r="E19" s="42" t="s">
+      <c r="E19" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F19" s="42"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="42"/>
-      <c r="I19" s="42"/>
-      <c r="J19" s="42"/>
-      <c r="K19" s="42"/>
-      <c r="L19" s="42"/>
-      <c r="M19" s="42"/>
-      <c r="N19" s="42"/>
-      <c r="O19" s="42" t="s">
+      <c r="F19" s="41"/>
+      <c r="G19" s="41"/>
+      <c r="H19" s="41"/>
+      <c r="I19" s="41"/>
+      <c r="J19" s="41"/>
+      <c r="K19" s="41"/>
+      <c r="L19" s="41"/>
+      <c r="M19" s="41"/>
+      <c r="N19" s="41"/>
+      <c r="O19" s="41" t="s">
         <v>609</v>
       </c>
-      <c r="P19" s="42" t="s">
+      <c r="P19" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q19" s="44" t="s">
+      <c r="Q19" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R19" s="42" t="s">
+      <c r="R19" s="41" t="s">
         <v>485</v>
       </c>
-      <c r="S19" s="42" t="s">
+      <c r="S19" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A20" s="42" t="s">
+      <c r="A20" s="41" t="s">
         <v>604</v>
       </c>
-      <c r="B20" s="42" t="s">
+      <c r="B20" s="41" t="s">
         <v>613</v>
       </c>
-      <c r="C20" s="42" t="s">
+      <c r="C20" s="41" t="s">
         <v>614</v>
       </c>
-      <c r="D20" s="43" t="s">
+      <c r="D20" s="42" t="s">
         <v>615</v>
       </c>
-      <c r="E20" s="42" t="s">
+      <c r="E20" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F20" s="42"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="42"/>
-      <c r="I20" s="42"/>
-      <c r="J20" s="42"/>
-      <c r="K20" s="42"/>
-      <c r="L20" s="42"/>
-      <c r="M20" s="42"/>
-      <c r="N20" s="42"/>
-      <c r="O20" s="42" t="s">
+      <c r="F20" s="41"/>
+      <c r="G20" s="41"/>
+      <c r="H20" s="41"/>
+      <c r="I20" s="41"/>
+      <c r="J20" s="41"/>
+      <c r="K20" s="41"/>
+      <c r="L20" s="41"/>
+      <c r="M20" s="41"/>
+      <c r="N20" s="41"/>
+      <c r="O20" s="41" t="s">
         <v>616</v>
       </c>
-      <c r="P20" s="42" t="s">
+      <c r="P20" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q20" s="44" t="s">
+      <c r="Q20" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R20" s="42" t="s">
+      <c r="R20" s="41" t="s">
         <v>486</v>
       </c>
-      <c r="S20" s="42" t="s">
+      <c r="S20" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A21" s="42" t="s">
+      <c r="A21" s="41" t="s">
         <v>604</v>
       </c>
-      <c r="B21" s="42" t="s">
+      <c r="B21" s="41" t="s">
         <v>617</v>
       </c>
-      <c r="C21" s="42" t="s">
+      <c r="C21" s="41" t="s">
         <v>618</v>
       </c>
-      <c r="D21" s="43" t="s">
+      <c r="D21" s="42" t="s">
         <v>619</v>
       </c>
-      <c r="E21" s="42" t="s">
+      <c r="E21" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F21" s="42"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="42"/>
-      <c r="I21" s="42"/>
-      <c r="J21" s="42"/>
-      <c r="K21" s="42"/>
-      <c r="L21" s="42"/>
-      <c r="M21" s="42"/>
-      <c r="N21" s="42"/>
-      <c r="O21" s="42" t="s">
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="41"/>
+      <c r="I21" s="41"/>
+      <c r="J21" s="41"/>
+      <c r="K21" s="41"/>
+      <c r="L21" s="41"/>
+      <c r="M21" s="41"/>
+      <c r="N21" s="41"/>
+      <c r="O21" s="41" t="s">
         <v>609</v>
       </c>
-      <c r="P21" s="42" t="s">
+      <c r="P21" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q21" s="44" t="s">
+      <c r="Q21" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R21" s="42" t="s">
+      <c r="R21" s="41" t="s">
         <v>487</v>
       </c>
-      <c r="S21" s="42" t="s">
+      <c r="S21" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A22" s="42" t="s">
+      <c r="A22" s="41" t="s">
         <v>620</v>
       </c>
-      <c r="B22" s="42" t="s">
+      <c r="B22" s="41" t="s">
         <v>621</v>
       </c>
-      <c r="C22" s="42" t="s">
+      <c r="C22" s="41" t="s">
         <v>622</v>
       </c>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="42" t="s">
         <v>623</v>
       </c>
-      <c r="E22" s="42" t="s">
+      <c r="E22" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="42"/>
-      <c r="J22" s="42"/>
-      <c r="K22" s="42"/>
-      <c r="L22" s="42"/>
-      <c r="M22" s="42"/>
-      <c r="N22" s="42"/>
-      <c r="O22" s="42" t="s">
+      <c r="F22" s="41"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="41"/>
+      <c r="J22" s="41"/>
+      <c r="K22" s="41"/>
+      <c r="L22" s="41"/>
+      <c r="M22" s="41"/>
+      <c r="N22" s="41"/>
+      <c r="O22" s="41" t="s">
         <v>616</v>
       </c>
-      <c r="P22" s="42" t="s">
+      <c r="P22" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q22" s="44" t="s">
+      <c r="Q22" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R22" s="42" t="s">
+      <c r="R22" s="41" t="s">
         <v>488</v>
       </c>
-      <c r="S22" s="42" t="s">
+      <c r="S22" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A23" s="42" t="s">
+      <c r="A23" s="41" t="s">
         <v>624</v>
       </c>
-      <c r="B23" s="42" t="s">
+      <c r="B23" s="41" t="s">
         <v>625</v>
       </c>
-      <c r="C23" s="42" t="s">
+      <c r="C23" s="41" t="s">
         <v>626</v>
       </c>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="42" t="s">
         <v>627</v>
       </c>
-      <c r="E23" s="42" t="s">
+      <c r="E23" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F23" s="42"/>
-      <c r="G23" s="42"/>
-      <c r="H23" s="42"/>
-      <c r="I23" s="42"/>
-      <c r="J23" s="42"/>
-      <c r="K23" s="42"/>
-      <c r="L23" s="42"/>
-      <c r="M23" s="42"/>
-      <c r="N23" s="42"/>
-      <c r="O23" s="42" t="s">
+      <c r="F23" s="41"/>
+      <c r="G23" s="41"/>
+      <c r="H23" s="41"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="41"/>
+      <c r="K23" s="41"/>
+      <c r="L23" s="41"/>
+      <c r="M23" s="41"/>
+      <c r="N23" s="41"/>
+      <c r="O23" s="41" t="s">
         <v>616</v>
       </c>
-      <c r="P23" s="42" t="s">
+      <c r="P23" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q23" s="44" t="s">
+      <c r="Q23" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R23" s="42" t="s">
+      <c r="R23" s="41" t="s">
         <v>489</v>
       </c>
-      <c r="S23" s="42" t="s">
+      <c r="S23" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A24" s="42" t="s">
+      <c r="A24" s="41" t="s">
         <v>628</v>
       </c>
-      <c r="B24" s="42" t="s">
+      <c r="B24" s="41" t="s">
         <v>629</v>
       </c>
-      <c r="C24" s="42" t="s">
+      <c r="C24" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="43" t="s">
+      <c r="D24" s="42" t="s">
         <v>630</v>
       </c>
-      <c r="E24" s="42"/>
-      <c r="F24" s="42"/>
-      <c r="G24" s="42"/>
-      <c r="H24" s="42"/>
-      <c r="I24" s="42"/>
-      <c r="J24" s="42"/>
-      <c r="K24" s="42"/>
-      <c r="L24" s="42"/>
-      <c r="M24" s="42"/>
-      <c r="N24" s="42"/>
-      <c r="O24" s="42" t="s">
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="41"/>
+      <c r="I24" s="41"/>
+      <c r="J24" s="41"/>
+      <c r="K24" s="41"/>
+      <c r="L24" s="41"/>
+      <c r="M24" s="41"/>
+      <c r="N24" s="41"/>
+      <c r="O24" s="41" t="s">
         <v>631</v>
       </c>
-      <c r="P24" s="42" t="s">
+      <c r="P24" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q24" s="44" t="s">
+      <c r="Q24" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R24" s="42" t="s">
+      <c r="R24" s="41" t="s">
         <v>632</v>
       </c>
-      <c r="S24" s="42" t="s">
+      <c r="S24" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A25" s="42" t="s">
+      <c r="A25" s="41" t="s">
         <v>633</v>
       </c>
-      <c r="B25" s="42" t="s">
+      <c r="B25" s="41" t="s">
         <v>634</v>
       </c>
-      <c r="C25" s="42" t="s">
+      <c r="C25" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="43" t="s">
+      <c r="D25" s="42" t="s">
         <v>635</v>
       </c>
-      <c r="E25" s="42" t="s">
+      <c r="E25" s="41" t="s">
         <v>513</v>
       </c>
-      <c r="F25" s="42"/>
-      <c r="G25" s="42"/>
-      <c r="H25" s="42"/>
-      <c r="I25" s="42"/>
-      <c r="J25" s="42"/>
-      <c r="K25" s="42"/>
-      <c r="L25" s="42"/>
-      <c r="M25" s="42"/>
-      <c r="N25" s="42"/>
-      <c r="O25" s="42" t="s">
+      <c r="F25" s="41"/>
+      <c r="G25" s="41"/>
+      <c r="H25" s="41"/>
+      <c r="I25" s="41"/>
+      <c r="J25" s="41"/>
+      <c r="K25" s="41"/>
+      <c r="L25" s="41"/>
+      <c r="M25" s="41"/>
+      <c r="N25" s="41"/>
+      <c r="O25" s="41" t="s">
         <v>493</v>
       </c>
-      <c r="P25" s="42" t="s">
+      <c r="P25" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q25" s="44" t="s">
+      <c r="Q25" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R25" s="42" t="s">
+      <c r="R25" s="41" t="s">
         <v>636</v>
       </c>
-      <c r="S25" s="42" t="s">
+      <c r="S25" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A26" s="42" t="s">
+      <c r="A26" s="41" t="s">
         <v>637</v>
       </c>
-      <c r="B26" s="42" t="s">
+      <c r="B26" s="41" t="s">
         <v>638</v>
       </c>
-      <c r="C26" s="42" t="s">
+      <c r="C26" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D26" s="43" t="s">
+      <c r="D26" s="42" t="s">
         <v>639</v>
       </c>
-      <c r="E26" s="42" t="s">
+      <c r="E26" s="41" t="s">
         <v>555</v>
       </c>
-      <c r="F26" s="42" t="s">
+      <c r="F26" s="41" t="s">
         <v>640</v>
       </c>
-      <c r="G26" s="42"/>
-      <c r="H26" s="42"/>
-      <c r="I26" s="42"/>
-      <c r="J26" s="42"/>
-      <c r="K26" s="42"/>
-      <c r="L26" s="42"/>
-      <c r="M26" s="42"/>
-      <c r="N26" s="42"/>
-      <c r="O26" s="42" t="s">
+      <c r="G26" s="41"/>
+      <c r="H26" s="41"/>
+      <c r="I26" s="41"/>
+      <c r="J26" s="41"/>
+      <c r="K26" s="41"/>
+      <c r="L26" s="41"/>
+      <c r="M26" s="41"/>
+      <c r="N26" s="41"/>
+      <c r="O26" s="41" t="s">
         <v>641</v>
       </c>
-      <c r="P26" s="42" t="s">
+      <c r="P26" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="Q26" s="44" t="s">
+      <c r="Q26" s="43" t="s">
         <v>557</v>
       </c>
-      <c r="R26" s="42" t="s">
+      <c r="R26" s="41" t="s">
         <v>642</v>
       </c>
-      <c r="S26" s="42" t="s">
+      <c r="S26" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A27" s="47" t="s">
+      <c r="A27" s="46" t="s">
         <v>637</v>
       </c>
-      <c r="B27" s="47" t="s">
+      <c r="B27" s="46" t="s">
         <v>643</v>
       </c>
-      <c r="C27" s="47" t="s">
+      <c r="C27" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="D27" s="48" t="s">
+      <c r="D27" s="47" t="s">
         <v>644</v>
       </c>
-      <c r="E27" s="47" t="s">
+      <c r="E27" s="46" t="s">
         <v>555</v>
       </c>
-      <c r="F27" s="47"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="47"/>
-      <c r="I27" s="47"/>
-      <c r="J27" s="47"/>
-      <c r="K27" s="47"/>
-      <c r="L27" s="47"/>
-      <c r="M27" s="47"/>
-      <c r="N27" s="47"/>
-      <c r="O27" s="47" t="s">
+      <c r="F27" s="46"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="46"/>
+      <c r="I27" s="46"/>
+      <c r="J27" s="46"/>
+      <c r="K27" s="46"/>
+      <c r="L27" s="46"/>
+      <c r="M27" s="46"/>
+      <c r="N27" s="46"/>
+      <c r="O27" s="46" t="s">
         <v>645</v>
       </c>
-      <c r="P27" s="47" t="s">
+      <c r="P27" s="46" t="s">
         <v>479</v>
       </c>
-      <c r="Q27" s="49" t="s">
+      <c r="Q27" s="48" t="s">
         <v>557</v>
       </c>
-      <c r="R27" s="47" t="s">
+      <c r="R27" s="46" t="s">
         <v>646</v>
       </c>
-      <c r="S27" s="47" t="s">
+      <c r="S27" s="46" t="s">
         <v>504</v>
       </c>
-      <c r="T27" s="50" t="s">
+      <c r="T27" s="49" t="s">
         <v>676</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A28" s="47" t="s">
+      <c r="A28" s="46" t="s">
         <v>647</v>
       </c>
-      <c r="B28" s="47" t="s">
+      <c r="B28" s="46" t="s">
         <v>648</v>
       </c>
-      <c r="C28" s="47" t="s">
+      <c r="C28" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="48" t="s">
+      <c r="D28" s="47" t="s">
         <v>649</v>
       </c>
-      <c r="E28" s="47" t="s">
+      <c r="E28" s="46" t="s">
         <v>555</v>
       </c>
-      <c r="F28" s="47" t="s">
+      <c r="F28" s="46" t="s">
         <v>650</v>
       </c>
-      <c r="G28" s="47" t="s">
+      <c r="G28" s="46" t="s">
         <v>651</v>
       </c>
-      <c r="H28" s="47" t="s">
+      <c r="H28" s="46" t="s">
         <v>652</v>
       </c>
-      <c r="I28" s="47" t="s">
+      <c r="I28" s="46" t="s">
         <v>653</v>
       </c>
-      <c r="J28" s="47" t="s">
+      <c r="J28" s="46" t="s">
         <v>654</v>
       </c>
-      <c r="K28" s="47" t="s">
+      <c r="K28" s="46" t="s">
         <v>655</v>
       </c>
-      <c r="L28" s="47" t="s">
+      <c r="L28" s="46" t="s">
         <v>656</v>
       </c>
-      <c r="M28" s="47" t="s">
+      <c r="M28" s="46" t="s">
         <v>657</v>
       </c>
-      <c r="N28" s="47" t="s">
+      <c r="N28" s="46" t="s">
         <v>658</v>
       </c>
-      <c r="O28" s="47" t="s">
+      <c r="O28" s="46" t="s">
         <v>645</v>
       </c>
-      <c r="P28" s="47" t="s">
+      <c r="P28" s="46" t="s">
         <v>479</v>
       </c>
-      <c r="Q28" s="49" t="s">
+      <c r="Q28" s="48" t="s">
         <v>557</v>
       </c>
-      <c r="R28" s="47" t="s">
+      <c r="R28" s="46" t="s">
         <v>659</v>
       </c>
-      <c r="S28" s="47" t="s">
+      <c r="S28" s="46" t="s">
         <v>504</v>
       </c>
-      <c r="T28" s="50" t="s">
+      <c r="T28" s="49" t="s">
         <v>675</v>
       </c>
     </row>
@@ -9016,22 +9049,22 @@
       <c r="U1" s="4"/>
     </row>
     <row r="2" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="51" t="s">
         <v>526</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="52" t="s">
         <v>526</v>
       </c>
-      <c r="C2" s="53" t="s">
+      <c r="C2" s="52" t="s">
         <v>479</v>
       </c>
-      <c r="D2" s="53" t="s">
+      <c r="D2" s="52" t="s">
         <v>527</v>
       </c>
-      <c r="E2" s="53" t="s">
+      <c r="E2" s="52" t="s">
         <v>528</v>
       </c>
-      <c r="F2" s="53" t="s">
+      <c r="F2" s="52" t="s">
         <v>504</v>
       </c>
       <c r="G2" s="4"/>
@@ -9051,20 +9084,20 @@
       <c r="U2" s="4"/>
     </row>
     <row r="3" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="52"/>
-      <c r="B3" s="53" t="s">
+      <c r="A3" s="51"/>
+      <c r="B3" s="52" t="s">
         <v>529</v>
       </c>
-      <c r="C3" s="53" t="s">
+      <c r="C3" s="52" t="s">
         <v>479</v>
       </c>
-      <c r="D3" s="53" t="s">
+      <c r="D3" s="52" t="s">
         <v>530</v>
       </c>
-      <c r="E3" s="53" t="s">
+      <c r="E3" s="52" t="s">
         <v>531</v>
       </c>
-      <c r="F3" s="53" t="s">
+      <c r="F3" s="52" t="s">
         <v>504</v>
       </c>
       <c r="O3" s="4"/>
@@ -9074,22 +9107,22 @@
       <c r="S3" s="4"/>
     </row>
     <row r="4" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="51" t="s">
         <v>513</v>
       </c>
-      <c r="B4" s="53" t="s">
+      <c r="B4" s="52" t="s">
         <v>529</v>
       </c>
-      <c r="C4" s="53" t="s">
+      <c r="C4" s="52" t="s">
         <v>479</v>
       </c>
-      <c r="D4" s="53" t="s">
+      <c r="D4" s="52" t="s">
         <v>532</v>
       </c>
-      <c r="E4" s="53" t="s">
+      <c r="E4" s="52" t="s">
         <v>533</v>
       </c>
-      <c r="F4" s="53" t="s">
+      <c r="F4" s="52" t="s">
         <v>504</v>
       </c>
       <c r="O4" s="4"/>
@@ -9099,7 +9132,7 @@
       <c r="S4" s="4"/>
     </row>
     <row r="5" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="50" t="s">
         <v>534</v>
       </c>
       <c r="B5" s="34" t="s">
@@ -9124,22 +9157,22 @@
       <c r="S5" s="4"/>
     </row>
     <row r="6" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="51" t="s">
         <v>538</v>
       </c>
-      <c r="B6" s="53" t="s">
+      <c r="B6" s="52" t="s">
         <v>538</v>
       </c>
-      <c r="C6" s="53" t="s">
+      <c r="C6" s="52" t="s">
         <v>479</v>
       </c>
-      <c r="D6" s="53" t="s">
+      <c r="D6" s="52" t="s">
         <v>539</v>
       </c>
-      <c r="E6" s="53" t="s">
+      <c r="E6" s="52" t="s">
         <v>540</v>
       </c>
-      <c r="F6" s="53" t="s">
+      <c r="F6" s="52" t="s">
         <v>504</v>
       </c>
       <c r="O6" s="4"/>
@@ -9149,22 +9182,22 @@
       <c r="S6" s="4"/>
     </row>
     <row r="7" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="52" t="s">
+      <c r="A7" s="51" t="s">
         <v>541</v>
       </c>
-      <c r="B7" s="53" t="s">
+      <c r="B7" s="52" t="s">
         <v>526</v>
       </c>
-      <c r="C7" s="53" t="s">
+      <c r="C7" s="52" t="s">
         <v>479</v>
       </c>
-      <c r="D7" s="53" t="s">
+      <c r="D7" s="52" t="s">
         <v>542</v>
       </c>
-      <c r="E7" s="53" t="s">
+      <c r="E7" s="52" t="s">
         <v>543</v>
       </c>
-      <c r="F7" s="53" t="s">
+      <c r="F7" s="52" t="s">
         <v>504</v>
       </c>
       <c r="O7" s="4"/>
@@ -9174,7 +9207,7 @@
       <c r="S7" s="4"/>
     </row>
     <row r="8" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="51">
+      <c r="A8" s="50">
         <v>1000000</v>
       </c>
       <c r="B8" s="34" t="s">
@@ -9199,7 +9232,7 @@
       <c r="S8" s="4"/>
     </row>
     <row r="9" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="51" t="s">
+      <c r="A9" s="50" t="s">
         <v>546</v>
       </c>
       <c r="B9" s="34" t="s">
@@ -9485,7 +9518,7 @@
       <c r="A2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="51"/>
+      <c r="B2" s="50"/>
       <c r="C2" s="34" t="s">
         <v>506</v>
       </c>
@@ -9509,7 +9542,7 @@
       <c r="A3" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="51">
+      <c r="B3" s="50">
         <v>123</v>
       </c>
       <c r="C3" s="34" t="s">
@@ -9538,7 +9571,7 @@
       <c r="A4" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="51" t="s">
+      <c r="B4" s="50" t="s">
         <v>513</v>
       </c>
       <c r="C4" s="34" t="s">
@@ -9564,7 +9597,7 @@
       <c r="A5" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="51" t="s">
+      <c r="B5" s="50" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="34" t="s">
@@ -9590,7 +9623,7 @@
       <c r="A6" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="51" t="s">
+      <c r="B6" s="50" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="34"/>
@@ -9614,7 +9647,7 @@
       <c r="A7" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="51" t="s">
+      <c r="B7" s="50" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="34" t="s">
@@ -9637,28 +9670,28 @@
       </c>
     </row>
     <row r="8" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="54" t="s">
+      <c r="A8" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="55" t="s">
+      <c r="B8" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="54" t="s">
+      <c r="C8" s="53" t="s">
         <v>506</v>
       </c>
-      <c r="D8" s="54" t="s">
+      <c r="D8" s="53" t="s">
         <v>522</v>
       </c>
-      <c r="E8" s="54" t="s">
+      <c r="E8" s="53" t="s">
         <v>479</v>
       </c>
-      <c r="F8" s="54" t="s">
+      <c r="F8" s="53" t="s">
         <v>523</v>
       </c>
-      <c r="G8" s="54" t="s">
+      <c r="G8" s="53" t="s">
         <v>524</v>
       </c>
-      <c r="H8" s="54" t="s">
+      <c r="H8" s="53" t="s">
         <v>504</v>
       </c>
     </row>
@@ -9738,227 +9771,227 @@
     </row>
     <row r="2" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="31"/>
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="41" t="s">
         <v>478</v>
       </c>
-      <c r="E2" s="42" t="s">
+      <c r="E2" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F2" s="42" t="s">
+      <c r="F2" s="41" t="s">
         <v>480</v>
       </c>
-      <c r="G2" s="42" t="s">
+      <c r="G2" s="41" t="s">
         <v>481</v>
       </c>
-      <c r="H2" s="42" t="s">
+      <c r="H2" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="31"/>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="44" t="s">
         <v>483</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F3" s="42" t="s">
+      <c r="F3" s="41" t="s">
         <v>480</v>
       </c>
-      <c r="G3" s="42" t="s">
+      <c r="G3" s="41" t="s">
         <v>484</v>
       </c>
-      <c r="H3" s="42" t="s">
+      <c r="H3" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="31"/>
-      <c r="D4" s="45" t="s">
+      <c r="D4" s="44" t="s">
         <v>483</v>
       </c>
-      <c r="E4" s="42" t="s">
+      <c r="E4" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F4" s="42" t="s">
+      <c r="F4" s="41" t="s">
         <v>480</v>
       </c>
-      <c r="G4" s="42" t="s">
+      <c r="G4" s="41" t="s">
         <v>485</v>
       </c>
-      <c r="H4" s="42" t="s">
+      <c r="H4" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="31"/>
-      <c r="D5" s="45" t="s">
+      <c r="D5" s="44" t="s">
         <v>483</v>
       </c>
-      <c r="E5" s="42" t="s">
+      <c r="E5" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F5" s="42" t="s">
+      <c r="F5" s="41" t="s">
         <v>480</v>
       </c>
-      <c r="G5" s="42" t="s">
+      <c r="G5" s="41" t="s">
         <v>486</v>
       </c>
-      <c r="H5" s="42" t="s">
+      <c r="H5" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="31"/>
-      <c r="D6" s="45" t="s">
+      <c r="D6" s="44" t="s">
         <v>483</v>
       </c>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F6" s="42" t="s">
+      <c r="F6" s="41" t="s">
         <v>480</v>
       </c>
-      <c r="G6" s="42" t="s">
+      <c r="G6" s="41" t="s">
         <v>487</v>
       </c>
-      <c r="H6" s="42" t="s">
+      <c r="H6" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D7" s="45" t="s">
+      <c r="D7" s="44" t="s">
         <v>483</v>
       </c>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F7" s="42" t="s">
+      <c r="F7" s="41" t="s">
         <v>480</v>
       </c>
-      <c r="G7" s="42" t="s">
+      <c r="G7" s="41" t="s">
         <v>488</v>
       </c>
-      <c r="H7" s="42" t="s">
+      <c r="H7" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D8" s="45" t="s">
+      <c r="D8" s="44" t="s">
         <v>483</v>
       </c>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F8" s="42" t="s">
+      <c r="F8" s="41" t="s">
         <v>480</v>
       </c>
-      <c r="G8" s="42" t="s">
+      <c r="G8" s="41" t="s">
         <v>489</v>
       </c>
-      <c r="H8" s="42" t="s">
+      <c r="H8" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D9" s="45" t="s">
+      <c r="D9" s="44" t="s">
         <v>490</v>
       </c>
-      <c r="E9" s="42" t="s">
+      <c r="E9" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F9" s="42" t="s">
+      <c r="F9" s="41" t="s">
         <v>491</v>
       </c>
-      <c r="G9" s="42" t="s">
+      <c r="G9" s="41" t="s">
         <v>492</v>
       </c>
-      <c r="H9" s="42" t="s">
+      <c r="H9" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D10" s="45" t="s">
+      <c r="D10" s="44" t="s">
         <v>493</v>
       </c>
-      <c r="E10" s="42" t="s">
+      <c r="E10" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F10" s="42" t="s">
+      <c r="F10" s="41" t="s">
         <v>491</v>
       </c>
-      <c r="G10" s="42" t="s">
+      <c r="G10" s="41" t="s">
         <v>494</v>
       </c>
-      <c r="H10" s="42" t="s">
+      <c r="H10" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D11" s="45" t="s">
+      <c r="D11" s="44" t="s">
         <v>493</v>
       </c>
-      <c r="E11" s="42" t="s">
+      <c r="E11" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F11" s="42" t="s">
+      <c r="F11" s="41" t="s">
         <v>491</v>
       </c>
-      <c r="G11" s="42" t="s">
+      <c r="G11" s="41" t="s">
         <v>495</v>
       </c>
-      <c r="H11" s="42" t="s">
+      <c r="H11" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D12" s="45" t="s">
+      <c r="D12" s="44" t="s">
         <v>496</v>
       </c>
-      <c r="E12" s="42" t="s">
+      <c r="E12" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F12" s="42" t="s">
+      <c r="F12" s="41" t="s">
         <v>491</v>
       </c>
-      <c r="G12" s="42" t="s">
+      <c r="G12" s="41" t="s">
         <v>497</v>
       </c>
-      <c r="H12" s="42" t="s">
+      <c r="H12" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D13" s="45" t="s">
+      <c r="D13" s="44" t="s">
         <v>496</v>
       </c>
-      <c r="E13" s="42" t="s">
+      <c r="E13" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F13" s="42" t="s">
+      <c r="F13" s="41" t="s">
         <v>491</v>
       </c>
-      <c r="G13" s="42" t="s">
+      <c r="G13" s="41" t="s">
         <v>498</v>
       </c>
-      <c r="H13" s="42" t="s">
+      <c r="H13" s="41" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D14" s="42" t="s">
+      <c r="D14" s="41" t="s">
         <v>499</v>
       </c>
-      <c r="E14" s="42" t="s">
+      <c r="E14" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F14" s="42" t="s">
+      <c r="F14" s="41" t="s">
         <v>491</v>
       </c>
-      <c r="G14" s="42" t="s">
+      <c r="G14" s="41" t="s">
         <v>500</v>
       </c>
-      <c r="H14" s="42" t="s">
+      <c r="H14" s="41" t="s">
         <v>482</v>
       </c>
       <c r="I14" s="25" t="s">
@@ -9966,19 +9999,19 @@
       </c>
     </row>
     <row r="15" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D15" s="42" t="s">
+      <c r="D15" s="41" t="s">
         <v>499</v>
       </c>
-      <c r="E15" s="42" t="s">
+      <c r="E15" s="41" t="s">
         <v>479</v>
       </c>
-      <c r="F15" s="42" t="s">
+      <c r="F15" s="41" t="s">
         <v>491</v>
       </c>
-      <c r="G15" s="42" t="s">
+      <c r="G15" s="41" t="s">
         <v>502</v>
       </c>
-      <c r="H15" s="42" t="s">
+      <c r="H15" s="41" t="s">
         <v>482</v>
       </c>
       <c r="I15" s="25" t="s">
@@ -9986,13 +10019,13 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D16" s="56"/>
-      <c r="E16" s="47" t="s">
+      <c r="D16" s="55"/>
+      <c r="E16" s="46" t="s">
         <v>479</v>
       </c>
-      <c r="F16" s="56"/>
-      <c r="G16" s="56"/>
-      <c r="H16" s="47" t="s">
+      <c r="F16" s="55"/>
+      <c r="G16" s="55"/>
+      <c r="H16" s="46" t="s">
         <v>504</v>
       </c>
     </row>
@@ -10067,161 +10100,161 @@
       </c>
     </row>
     <row r="2" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="57"/>
-      <c r="B2" s="58" t="s">
+      <c r="A2" s="56"/>
+      <c r="B2" s="57" t="s">
         <v>677</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57" t="s">
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56" t="s">
         <v>556</v>
       </c>
-      <c r="L2" s="57" t="s">
+      <c r="L2" s="56" t="s">
         <v>479</v>
       </c>
-      <c r="M2" s="57" t="s">
+      <c r="M2" s="56" t="s">
         <v>688</v>
       </c>
-      <c r="N2" s="59" t="s">
+      <c r="N2" s="58" t="s">
         <v>471</v>
       </c>
-      <c r="O2" s="57" t="s">
+      <c r="O2" s="56" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="56" t="s">
         <v>620</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="57" t="s">
+      <c r="B3" s="57"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="56"/>
+      <c r="K3" s="56" t="s">
         <v>590</v>
       </c>
-      <c r="L3" s="57" t="s">
+      <c r="L3" s="56" t="s">
         <v>479</v>
       </c>
-      <c r="M3" s="57" t="s">
+      <c r="M3" s="56" t="s">
         <v>688</v>
       </c>
-      <c r="N3" s="59" t="s">
+      <c r="N3" s="58" t="s">
         <v>472</v>
       </c>
-      <c r="O3" s="57" t="s">
+      <c r="O3" s="56" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="56" t="s">
         <v>620</v>
       </c>
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="57" t="s">
         <v>679</v>
       </c>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="57"/>
-      <c r="H4" s="57"/>
-      <c r="I4" s="57"/>
-      <c r="J4" s="57"/>
-      <c r="K4" s="57" t="s">
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="56" t="s">
         <v>593</v>
       </c>
-      <c r="L4" s="57" t="s">
+      <c r="L4" s="56" t="s">
         <v>479</v>
       </c>
-      <c r="M4" s="57" t="s">
+      <c r="M4" s="56" t="s">
         <v>688</v>
       </c>
-      <c r="N4" s="59" t="s">
+      <c r="N4" s="58" t="s">
         <v>473</v>
       </c>
-      <c r="O4" s="57" t="s">
+      <c r="O4" s="56" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="60" t="s">
+      <c r="A5" s="59" t="s">
         <v>620</v>
       </c>
-      <c r="B5" s="61" t="s">
+      <c r="B5" s="60" t="s">
         <v>677</v>
       </c>
-      <c r="C5" s="60" t="s">
+      <c r="C5" s="59" t="s">
         <v>651</v>
       </c>
-      <c r="D5" s="60" t="s">
+      <c r="D5" s="59" t="s">
         <v>681</v>
       </c>
-      <c r="E5" s="60" t="s">
+      <c r="E5" s="59" t="s">
         <v>680</v>
       </c>
-      <c r="F5" s="60" t="s">
+      <c r="F5" s="59" t="s">
         <v>682</v>
       </c>
-      <c r="G5" s="61" t="s">
+      <c r="G5" s="60" t="s">
         <v>683</v>
       </c>
-      <c r="H5" s="63" t="s">
+      <c r="H5" s="62" t="s">
         <v>684</v>
       </c>
-      <c r="I5" s="60" t="s">
+      <c r="I5" s="59" t="s">
         <v>685</v>
       </c>
-      <c r="J5" s="61" t="s">
+      <c r="J5" s="60" t="s">
         <v>686</v>
       </c>
-      <c r="K5" s="60" t="s">
+      <c r="K5" s="59" t="s">
         <v>687</v>
       </c>
-      <c r="L5" s="60" t="s">
+      <c r="L5" s="59" t="s">
         <v>479</v>
       </c>
-      <c r="M5" s="60" t="s">
+      <c r="M5" s="59" t="s">
         <v>688</v>
       </c>
-      <c r="N5" s="62" t="s">
+      <c r="N5" s="61" t="s">
         <v>474</v>
       </c>
-      <c r="O5" s="60" t="s">
+      <c r="O5" s="59" t="s">
         <v>504</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="60" t="s">
+      <c r="A6" s="59" t="s">
         <v>620</v>
       </c>
-      <c r="B6" s="61" t="s">
+      <c r="B6" s="60" t="s">
         <v>678</v>
       </c>
-      <c r="K6" s="60" t="s">
+      <c r="K6" s="59" t="s">
         <v>687</v>
       </c>
-      <c r="L6" s="60" t="s">
+      <c r="L6" s="59" t="s">
         <v>479</v>
       </c>
-      <c r="M6" s="60" t="s">
+      <c r="M6" s="59" t="s">
         <v>688</v>
       </c>
-      <c r="N6" s="62" t="s">
+      <c r="N6" s="61" t="s">
         <v>475</v>
       </c>
-      <c r="O6" s="60" t="s">
+      <c r="O6" s="59" t="s">
         <v>504</v>
       </c>
     </row>
@@ -10305,169 +10338,169 @@
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="57"/>
-      <c r="B2" s="58" t="s">
+      <c r="A2" s="56"/>
+      <c r="B2" s="57" t="s">
         <v>677</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57" t="s">
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56" t="s">
         <v>556</v>
       </c>
-      <c r="L2" s="57" t="s">
+      <c r="L2" s="56" t="s">
         <v>479</v>
       </c>
-      <c r="M2" s="57" t="s">
+      <c r="M2" s="56" t="s">
         <v>688</v>
       </c>
-      <c r="N2" s="59" t="s">
+      <c r="N2" s="58" t="s">
         <v>471</v>
       </c>
-      <c r="O2" s="57" t="s">
+      <c r="O2" s="56" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="56" t="s">
         <v>620</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="57" t="s">
+      <c r="B3" s="57"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="56"/>
+      <c r="K3" s="56" t="s">
         <v>590</v>
       </c>
-      <c r="L3" s="57" t="s">
+      <c r="L3" s="56" t="s">
         <v>479</v>
       </c>
-      <c r="M3" s="57" t="s">
+      <c r="M3" s="56" t="s">
         <v>688</v>
       </c>
-      <c r="N3" s="59" t="s">
+      <c r="N3" s="58" t="s">
         <v>472</v>
       </c>
-      <c r="O3" s="57" t="s">
+      <c r="O3" s="56" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="56" t="s">
         <v>620</v>
       </c>
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="57" t="s">
         <v>679</v>
       </c>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="57"/>
-      <c r="G4" s="57"/>
-      <c r="H4" s="57"/>
-      <c r="I4" s="57"/>
-      <c r="J4" s="57"/>
-      <c r="K4" s="57" t="s">
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="56" t="s">
         <v>593</v>
       </c>
-      <c r="L4" s="57" t="s">
+      <c r="L4" s="56" t="s">
         <v>479</v>
       </c>
-      <c r="M4" s="57" t="s">
+      <c r="M4" s="56" t="s">
         <v>688</v>
       </c>
-      <c r="N4" s="59" t="s">
+      <c r="N4" s="58" t="s">
         <v>473</v>
       </c>
-      <c r="O4" s="57" t="s">
+      <c r="O4" s="56" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="60" t="s">
+      <c r="A5" s="59" t="s">
         <v>620</v>
       </c>
-      <c r="B5" s="61" t="s">
+      <c r="B5" s="60" t="s">
         <v>677</v>
       </c>
-      <c r="C5" s="60"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="60"/>
-      <c r="F5" s="60"/>
-      <c r="G5" s="60"/>
-      <c r="H5" s="60"/>
-      <c r="I5" s="60"/>
-      <c r="J5" s="60"/>
-      <c r="K5" s="60" t="s">
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="59" t="s">
         <v>687</v>
       </c>
-      <c r="L5" s="60" t="s">
+      <c r="L5" s="59" t="s">
         <v>479</v>
       </c>
-      <c r="M5" s="60" t="s">
+      <c r="M5" s="59" t="s">
         <v>688</v>
       </c>
-      <c r="N5" s="62" t="s">
+      <c r="N5" s="61" t="s">
         <v>474</v>
       </c>
-      <c r="O5" s="60" t="s">
+      <c r="O5" s="59" t="s">
         <v>504</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="60" t="s">
+      <c r="A6" s="59" t="s">
         <v>620</v>
       </c>
-      <c r="B6" s="61" t="s">
+      <c r="B6" s="60" t="s">
         <v>678</v>
       </c>
-      <c r="C6" s="60" t="s">
+      <c r="C6" s="59" t="s">
         <v>651</v>
       </c>
-      <c r="D6" s="60" t="s">
+      <c r="D6" s="59" t="s">
         <v>681</v>
       </c>
-      <c r="E6" s="60" t="s">
+      <c r="E6" s="59" t="s">
         <v>680</v>
       </c>
-      <c r="F6" s="60" t="s">
+      <c r="F6" s="59" t="s">
         <v>682</v>
       </c>
-      <c r="G6" s="61" t="s">
+      <c r="G6" s="60" t="s">
         <v>683</v>
       </c>
-      <c r="H6" s="63" t="s">
+      <c r="H6" s="62" t="s">
         <v>684</v>
       </c>
-      <c r="I6" s="60" t="s">
+      <c r="I6" s="59" t="s">
         <v>685</v>
       </c>
-      <c r="J6" s="61" t="s">
+      <c r="J6" s="60" t="s">
         <v>686</v>
       </c>
-      <c r="K6" s="60" t="s">
+      <c r="K6" s="59" t="s">
         <v>687</v>
       </c>
-      <c r="L6" s="60" t="s">
+      <c r="L6" s="59" t="s">
         <v>479</v>
       </c>
-      <c r="M6" s="60" t="s">
+      <c r="M6" s="59" t="s">
         <v>688</v>
       </c>
-      <c r="N6" s="62" t="s">
+      <c r="N6" s="61" t="s">
         <v>475</v>
       </c>
-      <c r="O6" s="60" t="s">
+      <c r="O6" s="59" t="s">
         <v>504</v>
       </c>
     </row>
@@ -10603,7 +10636,7 @@
     <col min="10" max="10" width="9" style="21" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="9.140625" style="21" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="31.28515625" style="21" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.140625" style="64" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.140625" style="63" bestFit="1" customWidth="1"/>
     <col min="15" max="16384" width="9.140625" style="21"/>
   </cols>
   <sheetData>
@@ -10635,19 +10668,19 @@
       <c r="I1" s="24" t="s">
         <v>693</v>
       </c>
-      <c r="J1" s="64"/>
+      <c r="J1" s="63"/>
     </row>
     <row r="2" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
         <v>710</v>
       </c>
-      <c r="B2" s="68">
+      <c r="B2" s="67">
         <v>1</v>
       </c>
-      <c r="C2" s="67" t="s">
+      <c r="C2" s="66" t="s">
         <v>711</v>
       </c>
-      <c r="D2" s="66" t="s">
+      <c r="D2" s="65" t="s">
         <v>708</v>
       </c>
       <c r="E2" s="24" t="s">
@@ -10665,16 +10698,16 @@
       <c r="I2" s="24" t="s">
         <v>694</v>
       </c>
-      <c r="J2" s="64"/>
+      <c r="J2" s="63"/>
     </row>
     <row r="3" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="68">
+      <c r="B3" s="67">
         <v>1</v>
       </c>
-      <c r="C3" s="67" t="s">
+      <c r="C3" s="66" t="s">
         <v>712</v>
       </c>
-      <c r="D3" s="66" t="s">
+      <c r="D3" s="65" t="s">
         <v>708</v>
       </c>
       <c r="E3" s="24" t="s">
@@ -10692,19 +10725,19 @@
       <c r="I3" s="24" t="s">
         <v>695</v>
       </c>
-      <c r="J3" s="64"/>
+      <c r="J3" s="63"/>
     </row>
     <row r="4" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="21" t="s">
         <v>526</v>
       </c>
-      <c r="B4" s="68">
+      <c r="B4" s="67">
         <v>5</v>
       </c>
-      <c r="C4" s="67" t="s">
+      <c r="C4" s="66" t="s">
         <v>713</v>
       </c>
-      <c r="D4" s="66" t="s">
+      <c r="D4" s="65" t="s">
         <v>708</v>
       </c>
       <c r="E4" s="24" t="s">
@@ -10722,7 +10755,7 @@
       <c r="I4" s="24" t="s">
         <v>696</v>
       </c>
-      <c r="J4" s="64"/>
+      <c r="J4" s="63"/>
     </row>
     <row r="5" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I5" s="20"/>
@@ -10767,7 +10800,7 @@
     <row r="42" spans="14:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="43" spans="14:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="44" spans="14:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="N44" s="65" t="s">
+      <c r="N44" s="64" t="s">
         <v>457</v>
       </c>
     </row>

</xml_diff>